<commit_message>
Complete CBT exam engine with auto submit and result system
</commit_message>
<xml_diff>
--- a/AIAPGET_Questions.xlsx
+++ b/AIAPGET_Questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,252 +545,252 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Agadatantra</t>
+          <t>Dravyaguna</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>In the context of legal death investigations (inquests), which of the official figures shown in the image is typically responsible for performing the medical dissection and clinical autopsy to determine the scientific cause of death?</t>
+          <t>Amalaki has which rasa?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sub-Inspector of Police</t>
+          <t>Madhura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Executive Magistrate</t>
+          <t>Amla</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Forensic Pathologist</t>
+          <t>Tikta</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Insurance Investigator</t>
+          <t>Katu</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Forensic Pathologist</t>
+          <t>Amla</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>A Forensic Pathologist is a specially trained medical doctor who performs autopsies (post-mortem examinations). Their role within an inquest is to examine the body, document physical injuries, run toxicology tests, and provide expert medical evidence regarding the exact scientific cause and mechanism of death.</t>
+          <t>Amalaki is predominantly Amla rasa.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dravyaguna</t>
+          <t>Kaumarabhritya</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Amalaki has which rasa?</t>
+          <t>Kaumarabhritya deals with?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Madhura</t>
+          <t>Children</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Amla</t>
+          <t>Adults</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tikta</t>
+          <t>Elderly</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Katu</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Amla</t>
+          <t>Children</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Amalaki is predominantly Amla rasa.</t>
+          <t>It is pediatrics.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kaumarabhritya</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kaumarabhritya deals with?</t>
+          <t>Vata is composed of?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Children</t>
+          <t>Agni</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Adults</t>
+          <t>Vayu + Akasha</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Elderly</t>
+          <t>Jala</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Prithvi</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Children</t>
+          <t>Vayu + Akasha</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>It is pediatrics.</t>
+          <t>Vata is formed by Vayu and Akasha.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>Kriya Sharira</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vata is composed of?</t>
+          <t>Pitta is mainly responsible for?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Agni</t>
+          <t>Movement</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Vayu + Akasha</t>
+          <t>Digestion</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Jala</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Prithvi</t>
+          <t>Lubrication</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Vayu + Akasha</t>
+          <t>Digestion</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Vata is formed by Vayu and Akasha.</t>
+          <t>Pitta governs digestion and metabolism.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kriya Sharira</t>
+          <t>Modern Topics</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pitta is mainly responsible for?</t>
+          <t>WHO stands for?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Movement</t>
+          <t>World Health Organization</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Digestion</t>
+          <t>World Human Org</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Health World Org</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Lubrication</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Digestion</t>
+          <t>World Health Organization</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Pitta governs digestion and metabolism.</t>
+          <t>WHO is global health body.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Modern Topics</t>
+          <t>Padartha VIjnana</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>WHO stands for?</t>
+          <t>विवर्त वाद IS ACCEPTE BY</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>World Health Organization</t>
+          <t>जैन</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>World Human Org</t>
+          <t>वैशेषिक</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Health World Org</t>
+          <t>चार्वाक</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>वेदान्त</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>World Health Organization</t>
+          <t>वेदान्त</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>WHO is global health body.</t>
+          <t>SEE BOOK</t>
         </is>
       </c>
     </row>
@@ -802,32 +802,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>विवर्त वाद IS ACCEPTE BY</t>
+          <t>IN सृष्टि उत्पत्ति, नप्रकृति न विकृति IS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>अहंकार</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>पुरुष</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>चार्वाक</t>
+          <t>महत्</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>मनस्</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>पुरुष</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -844,32 +844,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IN सृष्टि उत्पत्ति, नप्रकृति न विकृति IS</t>
+          <t>ACCORDING TO कारिकावलि, THE सामान्य WHICH PERVADES ALL द्रव्य, गुण , कर्म IS CALLED AS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>अहंकार</t>
+          <t>परसामान्य</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>अपरसामान्य</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>महत्</t>
+          <t xml:space="preserve">परापरसामान्य </t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>मनस्</t>
+          <t>विशेषसामन्य</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>परसामान्य</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -886,32 +886,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ACCORDING TO कारिकावलि, THE सामान्य WHICH PERVADES ALL द्रव्य, गुण , कर्म IS CALLED AS</t>
+          <t>THE अभाव WHICH IS BOTH  आदि AND अनन्त IS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>परसामान्य</t>
+          <t>प्राग्भाव</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>अपरसामान्य</t>
+          <t>प्रध्वंसाभाव</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">परापरसामान्य </t>
+          <t>अन्योन्याभाव</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>विशेषसामन्य</t>
+          <t>सर्वाभाव</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>परसामान्य</t>
+          <t>अन्योन्याभाव</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -928,32 +928,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>THE अभाव WHICH IS BOTH  आदि AND अनन्त IS</t>
+          <t>IN अनुमान, परामर्श WILL EVOLVE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>प्राग्भाव</t>
+          <t>AFTER ESTABLISHMENT OF व्याप्ति</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>प्रध्वंसाभाव</t>
+          <t>BEFORE व्याप्ति</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>अन्योन्याभाव</t>
+          <t>AFTER पक्षधर्मत</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>सर्वाभाव</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>अन्योन्याभाव</t>
+          <t>AFTER पक्षधर्मत</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -970,32 +970,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IN अनुमान, परामर्श WILL EVOLVE</t>
+          <t>THE STATEMENT, पृथ्वि IS DIFFERENT FROM OTHER भूतs BECAUSE THEY DONT HAVE गन्धगुण IS AN EXAMPLE OF</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AFTER ESTABLISHMENT OF व्याप्ति</t>
+          <t>केवलान्वयि</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BEFORE व्याप्ति</t>
+          <t>केवलव्यतिरेकि</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>AFTER पक्षधर्मत</t>
+          <t xml:space="preserve">BOTH </t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>विशेष व्यतिरेकि</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>AFTER पक्षधर्मत</t>
+          <t>केवलव्यतिरेकि</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1012,32 +1012,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>THE STATEMENT, पृथ्वि IS DIFFERENT FROM OTHER भूतs BECAUSE THEY DONT HAVE गन्धगुण IS AN EXAMPLE OF</t>
+          <t>धर्म, अधर्म ARE पदार्थ/DRAVYA ACCORDING TO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>केवलान्वयि</t>
+          <t>सांख्य</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>केवलव्यतिरेकि</t>
+          <t>जैन</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOTH </t>
+          <t>वेदान्त</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>विशेष व्यतिरेकि</t>
+          <t>बौद्ध</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>केवलव्यतिरेकि</t>
+          <t>जैन</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1054,32 +1054,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>धर्म, अधर्म ARE पदार्थ/DRAVYA ACCORDING TO</t>
+          <t>विशिष्टाद्वैत POPULARISED BY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>सांख्य</t>
+          <t>रामानुजाचार्य</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>शंकराचार्य</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>मध्वाचार्य</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>बौद्ध</t>
+          <t>प्रभाकर</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>रामानुजाचार्य</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1096,32 +1096,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>विशिष्टाद्वैत POPULARISED BY</t>
+          <t>चेष्टा प्रमाण IS ACCEPTED BY</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>रामानुजाचार्य</t>
+          <t>प्रभाकर मीमांस</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>शंकराचार्य</t>
+          <t>पौराणिक</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>मध्वाचार्य</t>
+          <t>तान्त्रिक</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>प्रभाकर</t>
+          <t>मध्व</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>रामानुजाचार्य</t>
+          <t>तान्त्रिक</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1138,32 +1138,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>चेष्टा प्रमाण IS ACCEPTED BY</t>
+          <t>FROM WHICH दर्शन AYURVEDA TAKEN षट् पदार्थ</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>प्रभाकर मीमांस</t>
+          <t xml:space="preserve">सांख्य </t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>पौराणिक</t>
+          <t>योग</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>तान्त्रिक</t>
+          <t>न्याय</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>मध्व</t>
+          <t>वैशेषिक</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>तान्त्रिक</t>
+          <t>वैशेषिक</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1180,32 +1180,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FROM WHICH दर्शन AYURVEDA TAKEN षट् पदार्थ</t>
+          <t>ACCORDING TO चरक अतिवाहिक पुरुष IS NOT ASSOCIATED WITH</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">सांख्य </t>
+          <t>मन</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>योग</t>
+          <t xml:space="preserve">मन- आकाश       </t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>न्याय</t>
+          <t>इन्द्रिय</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>इन्द्रिय</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1222,32 +1222,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ACCORDING TO चरक अतिवाहिक पुरुष IS NOT ASSOCIATED WITH</t>
+          <t>षट् पदार्थ ARE CALLED BY चरक AS</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>मन</t>
+          <t>कार्य</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">मन- आकाश       </t>
+          <t>पदार्थ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>इन्द्रिय</t>
+          <t>कारण</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>विशेष</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>इन्द्रिय</t>
+          <t>कारण</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1264,32 +1264,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>षट् पदार्थ ARE CALLED BY चरक AS</t>
+          <t>WHICH इन्द्रिय प्रत्यक्ष प्रमाण NOT USED TO EXAMINE रोगि</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>कार्य</t>
+          <t>स्पर्शनेन्द्रिय</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>पदार्थ</t>
+          <t xml:space="preserve">चक्षुरेन्द्रिय </t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>रस्नेन्द्रिय</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>विशेष</t>
+          <t>घ्राणेन्द्रिय</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>रस्नेन्द्रिय</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1306,32 +1306,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>WHICH इन्द्रिय प्रत्यक्ष प्रमाण NOT USED TO EXAMINE रोगि</t>
+          <t>यस्य विवरणे शक्ति: IS</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>स्पर्शनेन्द्रिय</t>
+          <t>खर</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">चक्षुरेन्द्रिय </t>
+          <t xml:space="preserve">द्रव </t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>रस्नेन्द्रिय</t>
+          <t xml:space="preserve">सूक्ष्म       </t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>घ्राणेन्द्रिय</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>रस्नेन्द्रिय</t>
+          <t>सूक्ष्म</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1348,32 +1348,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>यस्य विवरणे शक्ति: IS</t>
+          <t>THE ELASTICITY OF RUBBER IS AN EXAMPLE FOR</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>खर</t>
+          <t xml:space="preserve">वेगाख्य संस्कार </t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">द्रव </t>
+          <t>स्थितिस्थापक</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">सूक्ष्म       </t>
+          <t>प्रतिविरुद्ध</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>भावनाख्य संस्कार</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>सूक्ष्म</t>
+          <t>स्थितिस्थापक</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1390,32 +1390,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>THE ELASTICITY OF RUBBER IS AN EXAMPLE FOR</t>
+          <t>FOLLOWING IS NOT THE USE OF काल</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">वेगाख्य संस्कार </t>
+          <t>DRUG ADMINISTRATION</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>स्थितिस्थापक</t>
+          <t>KNOWING DISESE STATUS</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>प्रतिविरुद्ध</t>
+          <t xml:space="preserve">KNOWING SEASONS      </t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>भावनाख्य संस्कार</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>स्थितिस्थापक</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1432,32 +1432,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FOLLOWING IS NOT THE USE OF काल</t>
+          <t>अविनावभाव सम्बन्ध IS</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DRUG ADMINISTRATION</t>
+          <t>सामान्यतो दॄष्ट अनुमान</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KNOWING DISESE STATUS</t>
+          <t>अन्वयव्यतिरेकि</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">KNOWING SEASONS      </t>
+          <t>कल्पना</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>व्याप्ति</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>व्याप्ति</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1469,615 +1469,615 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Padartha Vijnana</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>अविनावभाव सम्बन्ध IS</t>
+          <t>Dravya means?</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>सामान्यतो दॄष्ट अनुमान</t>
+          <t>Substance</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>अन्वयव्यतिरेकि</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>कल्पना</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>व्याप्ति</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>व्याप्ति</t>
+          <t>Substance</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>Dravya refers to substance.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Panchakarma</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>विवर्त वाद IS ACCEPTE BY</t>
+          <t>Vamana is?</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>Emesis</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>Purgation</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>चार्वाक</t>
+          <t>Enema</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>Nasal therapy</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>Emesis</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>Vamana is therapeutic emesis.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Prasooti Tantra &amp; Stree Roga</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IN सृष्टि उत्पत्ति, नप्रकृति न विकृति IS</t>
+          <t>Garbhini means?</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>अहंकार</t>
+          <t>Pregnant woman</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>Child</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>महत्</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>मनस्</t>
+          <t>Nurse</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>Pregnant woman</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>Garbhini refers to pregnant woman.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ACCORDING TO कारिकावलि, THE सामान्य WHICH PERVADES ALL द्रव्य, गुण , कर्म IS CALLED AS</t>
+          <t>Number of bones in adult human body?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>परसामान्य</t>
+          <t>206</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>अपरसामान्य</t>
+          <t>210</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">परापरसामान्य </t>
+          <t>300</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>विशेषसामन्य</t>
+          <t>180</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>परसामान्य</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>Adult human body has 206 bones.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>THE अभाव WHICH IS BOTH  आदि AND अनन्त IS</t>
+          <t>Parada is?</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>प्राग्भाव</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>प्रध्वंसाभाव</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>अन्योन्याभाव</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>सर्वाभाव</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>अन्योन्याभाव</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>Parada refers to mercury.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Research Methodology &amp; Statistics</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>IN अनुमान, परामर्श WILL EVOLVE</t>
+          <t>Mean is?</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AFTER ESTABLISHMENT OF व्याप्ति</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>BEFORE व्याप्ति</t>
+          <t>Median</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AFTER पक्षधर्मत</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>AFTER पक्षधर्मत</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>Mean is average.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Roganidana</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>THE STATEMENT, पृथ्वि IS DIFFERENT FROM OTHER भूतs BECAUSE THEY DONT HAVE गन्धगुण IS AN EXAMPLE OF</t>
+          <t>Nidana means?</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>केवलान्वयि</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>केवलव्यतिरेकि</t>
+          <t>Treatment</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOTH </t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>विशेष व्यतिरेकि</t>
+          <t>Exercise</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>केवलव्यतिरेकि</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>Nidana refers to diagnosis.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>धर्म, अधर्म ARE पदार्थ/DRAVYA ACCORDING TO</t>
+          <t>Charaka Samhita belongs to?</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>सांख्य</t>
+          <t>Shalya</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>Shalakya</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>बौद्ध</t>
+          <t>Kaumarabhritya</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>विशिष्टाद्वैत POPULARISED BY</t>
+          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>रामानुजाचार्य</t>
+          <t>तैल</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>शंकराचार्य</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>मध्वाचार्य</t>
+          <t>वसा</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>प्रभाकर</t>
+          <t>मज्जा</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>रामानुजाचार्य</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>चेष्टा प्रमाण IS ACCEPTED BY</t>
+          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>प्रभाकर मीमांस</t>
+          <t>शिशिर</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>पौराणिक</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>तान्त्रिक</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>मध्व</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>तान्त्रिक</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>FROM WHICH दर्शन AYURVEDA TAKEN षट् पदार्थ</t>
+          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">सांख्य </t>
+          <t>शब्दकल्पद्रुम</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>योग</t>
+          <t>तत्वचन्द्रिक</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>न्याय</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>न्यायचन्द्रिक</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ACCORDING TO चरक अतिवाहिक पुरुष IS NOT ASSOCIATED WITH</t>
+          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>मन</t>
+          <t>चरक</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">मन- आकाश       </t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>इन्द्रिय</t>
+          <t>अग्निवेश</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>नागार्जुन</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>इन्द्रिय</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>षट् पदार्थ ARE CALLED BY चरक AS</t>
+          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>कार्य</t>
+          <t>इंन्द्र</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>पदार्थ</t>
+          <t>सहस्राक्ष</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>प्रजापति</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>विशेष</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>WHICH इन्द्रिय प्रत्यक्ष प्रमाण NOT USED TO EXAMINE रोगि</t>
+          <t>भिन्नक्रम IS A</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>स्पर्शनेन्द्रिय</t>
+          <t>तन्त्रयुक्ति</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">चक्षुरेन्द्रिय </t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>रस्नेन्द्रिय</t>
+          <t>BOTH</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>घ्राणेन्द्रिय</t>
+          <t>तन्त्रगुण</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>रस्नेन्द्रिय</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>यस्य विवरणे शक्ति: IS</t>
+          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>खर</t>
+          <t>अध्यायन</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">द्रव </t>
+          <t>अध्यापन</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">सूक्ष्म       </t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2087,474 +2087,474 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>सूक्ष्म</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>THE ELASTICITY OF RUBBER IS AN EXAMPLE FOR</t>
+          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">वेगाख्य संस्कार </t>
+          <t>34</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>स्थितिस्थापक</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>प्रतिविरुद्ध</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>भावनाख्य संस्कार</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>स्थितिस्थापक</t>
+          <t>36</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>FOLLOWING IS NOT THE USE OF काल</t>
+          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DRUG ADMINISTRATION</t>
+          <t>एकदोषज</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>KNOWING DISESE STATUS</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">KNOWING SEASONS      </t>
+          <t>त्रिदोषज</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>वातज</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>अविनावभाव सम्बन्ध IS</t>
+          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>सामान्यतो दॄष्ट अनुमान</t>
+          <t>अष्टांग हृदय</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>अन्वयव्यतिरेकि</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>कल्पना</t>
+          <t>सुश्रुत संहिता</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>व्याप्ति</t>
+          <t>अष्टांग संग्रह</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>व्याप्ति</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Padartha Vijnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dravya means?</t>
+          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Substance</t>
+          <t>पिप्पलि</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Quality</t>
+          <t>अपमार्ग</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>नीलिनी</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Substance</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Dravya refers to substance.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Padartha Vijnana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>IDENTIFY THE IMAGE WITH RESPECT TO अभाव</t>
+          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>प्राग्भाव</t>
+          <t>वसन्त</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>अत्यन्ताभाव</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>प्रध्वम्साभाव</t>
+          <t>शरत्</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>प्रध्वम्साभाव</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>BROKEN POT</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Panchakarma</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Vamana is?</t>
+          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Emesis</t>
+          <t>NORTH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Purgation</t>
+          <t>SOUTH</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Enema</t>
+          <t>EAST</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Nasal therapy</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Emesis</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Vamana is therapeutic emesis.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Prasooti Tantra &amp; Stree Roga</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Garbhini means?</t>
+          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Pregnant woman</t>
+          <t>मधुर</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Child</t>
+          <t>आम्ल</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Nurse</t>
+          <t>तिक्त</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Pregnant woman</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Garbhini refers to pregnant woman.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Rachana Sharira</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Number of bones in adult human body?</t>
+          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>84</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>72</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>108</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Adult human body has 206 bones.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Parada is?</t>
+          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>COPPERISH</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Parada refers to mercury.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Research Methodology &amp; Statistics</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Mean is?</t>
+          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>तिर्यक्दोष</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Median</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>अनुपस्थितदोश</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>ऊर्ध्वदोष</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Mean is average.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Roganidana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Nidana means?</t>
+          <t>अवपीडक सर्पि IS GIVEN IN</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>छर्दिवेगधारण</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Treatment</t>
+          <t>पुरिषवेगधारण</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Exercise</t>
+          <t>अश्रुवेगधारण</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Nidana refers to diagnosis.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
@@ -2566,37 +2566,37 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Charaka Samhita belongs to?</t>
+          <t>WHICH IS RIGHT</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Shalya</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Shalakya</t>
+          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Kaumarabhritya</t>
+          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
@@ -2608,32 +2608,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
+          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>तैल</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>ABUNDANT AVAILABILIT</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>वसा</t>
+          <t>SHOULD HAVE MORE PARTS</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>मज्जा</t>
+          <t>MULTIPLE COLORS</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2650,32 +2650,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
+          <t>सुरा IS IDEAL अनुपान FOR</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>शिशिर</t>
+          <t>स्थूल</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>शोष</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>विष</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2692,32 +2692,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
+          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>शब्दकल्पद्रुम</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>तत्वचन्द्रिक</t>
+          <t>कांस्य</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>स्वर्णा</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>न्यायचन्द्रिक</t>
+          <t>मुक्ता</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2734,32 +2734,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
+          <t>वात प्रकोप IS CAUSED BY</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>चरक</t>
+          <t>उष्ण युक्त रूक्ष</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>अग्निवेश</t>
+          <t>शीत युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>नागार्जुन</t>
+          <t>उष्ण युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2776,32 +2776,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
+          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>इंन्द्र</t>
+          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>सहस्राक्ष</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>प्रजापति</t>
+          <t>कर्ममिथ्यायोग</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>वाक् मिथ्यायोग</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2818,32 +2818,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>भिन्नक्रम IS A</t>
+          <t>दूषिकI  IS मल OF</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>तन्त्रयुक्ति</t>
+          <t>कर्ण</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>नास</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>BOTH</t>
+          <t>आस्य</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>तन्त्रगुण</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2855,1048 +2855,250 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Samhita Adhyayana 2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
+          <t>Sushruta is known for?</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>अध्यायन</t>
+          <t>Medicine</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>अध्यापन</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>Toxicology</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Sushruta is father of surgery.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Samhita Adhyayana 3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
+          <t>Ashtanga Hridaya written by?</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>Charaka</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>Sushruta</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>Kashyapa</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Vagbhata authored Ashtanga Hridaya.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Sanskrit</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
+          <t>Meaning of 'Vaidya'?</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>एकदोषज</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>त्रिदोषज</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>वातज</t>
+          <t>King</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Vaidya means physician.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Shalakya Tantra</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
+          <t>Shalakya deals with?</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>अष्टांग हृदय</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>सुश्रुत संहिता</t>
+          <t>Bones</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>अष्टांग संग्रह</t>
+          <t>Skin</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>It deals with Urdhwajatrugata rogas.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Shalya Tantra</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
+          <t>Shalya Tantra deals with?</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>पिप्पलि</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>अपमार्ग</t>
+          <t>Medicine</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>नीलिनी</t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Shalya Tantra is surgical branch.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Swasthavritta</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
+          <t>Dinacharya refers to?</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>वसन्त</t>
+          <t>Daily routine</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>Night routine</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>शरत्</t>
+          <t>Seasonal routine</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>Daily routine</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>NORTH</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>SOUTH</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>EAST</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>WEST</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>WEST</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>मधुर</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>आम्ल</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>लवण</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>तिक्त</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>लवण</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>108</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>BLUE</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>YELLOW</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>COPPERISH</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>तिर्यक्दोष</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>उपस्थितदोष</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>अनुपस्थितदोश</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>ऊर्ध्वदोष</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>उपस्थितदोष</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>अवपीडक सर्पि IS GIVEN IN</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>छर्दिवेगधारण</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>पुरिषवेगधारण</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>मूत्रवेगधारण</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>अश्रुवेगधारण</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>मूत्रवेगधारण</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>WHICH IS RIGHT</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>MULTIPLE PROPERTY</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>ABUNDANT AVAILABILIT</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>SHOULD HAVE MORE PARTS</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>MULTIPLE COLORS</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>MULTIPLE PROPERTY</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>सुरा IS IDEAL अनुपान FOR</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>स्थूल</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>कृश</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>शोष</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>विष</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>कृश</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>रजत</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>कांस्य</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>स्वर्णा</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>मुक्ता</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>रजत</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>वात प्रकोप IS CAUSED BY</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>उष्ण युक्त रूक्ष</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>शीत युक्त रूक्ष</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>शीत युक्त स्निग्ध</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>उष्ण युक्त स्निग्ध</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>शीत युक्त रूक्ष</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>कर्ममिथ्यायोग</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>वाक् मिथ्यायोग</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 1</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>दूषिकI  IS मल OF</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>कर्ण</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>नास</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>आस्य</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>नेत्र</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>नेत्र</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>REFER BOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 2</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Sushruta is known for?</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Medicine</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Surgery</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Pediatrics</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Toxicology</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Surgery</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>Sushruta is father of surgery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Samhita Adhyayana 3</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Ashtanga Hridaya written by?</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Charaka</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Sushruta</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Vagbhata</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>Kashyapa</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Vagbhata</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>Vagbhata authored Ashtanga Hridaya.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Sanskrit</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Meaning of 'Vaidya'?</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Doctor</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Teacher</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Student</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>King</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>Doctor</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>Vaidya means physician.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Shalakya Tantra</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Shalakya deals with?</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>ENT &amp; Eye</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Heart</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Bones</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>Skin</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>ENT &amp; Eye</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>It deals with Urdhwajatrugata rogas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Shalya Tantra</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Shalya Tantra deals with?</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Surgery</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Medicine</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Pediatrics</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Diet</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>Surgery</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>Shalya Tantra is surgical branch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Swasthavritta</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Dinacharya refers to?</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>Daily routine</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Night routine</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Seasonal routine</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>Daily routine</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
         <is>
           <t>Dinacharya means daily regimen.</t>
         </is>

</xml_diff>

<commit_message>
Added student dashboard with analytics
</commit_message>
<xml_diff>
--- a/AIAPGET_Questions.xlsx
+++ b/AIAPGET_Questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1469,294 +1469,294 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Padartha Vijnana</t>
+          <t>Panchakarma</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dravya means?</t>
+          <t>Vamana is?</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Substance</t>
+          <t>Emesis</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Quality</t>
+          <t>Purgation</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Enema</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Nasal therapy</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Substance</t>
+          <t>Emesis</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Dravya refers to substance.</t>
+          <t>Vamana is therapeutic emesis.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Panchakarma</t>
+          <t>Prasooti Tantra &amp; Stree Roga</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Vamana is?</t>
+          <t>Garbhini means?</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Emesis</t>
+          <t>Pregnant woman</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Purgation</t>
+          <t>Child</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Enema</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Nasal therapy</t>
+          <t>Nurse</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Emesis</t>
+          <t>Pregnant woman</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Vamana is therapeutic emesis.</t>
+          <t>Garbhini refers to pregnant woman.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Prasooti Tantra &amp; Stree Roga</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Garbhini means?</t>
+          <t>Number of bones in adult human body?</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pregnant woman</t>
+          <t>206</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Child</t>
+          <t>210</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>300</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Nurse</t>
+          <t>180</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Pregnant woman</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Garbhini refers to pregnant woman.</t>
+          <t>Adult human body has 206 bones.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rachana Sharira</t>
+          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Number of bones in adult human body?</t>
+          <t>Parada is?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Adult human body has 206 bones.</t>
+          <t>Parada refers to mercury.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
+          <t>Research Methodology &amp; Statistics</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Parada is?</t>
+          <t>Mean is?</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Median</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Parada refers to mercury.</t>
+          <t>Mean is average.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Research Methodology &amp; Statistics</t>
+          <t>Roganidana</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mean is?</t>
+          <t>Nidana means?</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Median</t>
+          <t>Treatment</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Exercise</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Mean is average.</t>
+          <t>Nidana refers to diagnosis.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Roganidana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nidana means?</t>
+          <t>Charaka Samhita belongs to?</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>Shalya</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Treatment</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>Shalakya</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Exercise</t>
+          <t>Kaumarabhritya</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Nidana refers to diagnosis.</t>
+          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
         </is>
       </c>
     </row>
@@ -1768,37 +1768,37 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Charaka Samhita belongs to?</t>
+          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Shalya</t>
+          <t>तैल</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Shalakya</t>
+          <t>वसा</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Kaumarabhritya</t>
+          <t>मज्जा</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
@@ -1810,32 +1810,32 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
+          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>तैल</t>
+          <t>शिशिर</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>वसा</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>मज्जा</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1852,32 +1852,32 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
+          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>शिशिर</t>
+          <t>शब्दकल्पद्रुम</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>तत्वचन्द्रिक</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>न्यायचन्द्रिक</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1894,32 +1894,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
+          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>शब्दकल्पद्रुम</t>
+          <t>चरक</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>तत्वचन्द्रिक</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>अग्निवेश</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>न्यायचन्द्रिक</t>
+          <t>नागार्जुन</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1936,32 +1936,32 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
+          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>चरक</t>
+          <t>इंन्द्र</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>सहस्राक्ष</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>अग्निवेश</t>
+          <t>प्रजापति</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>नागार्जुन</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1978,32 +1978,32 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
+          <t>भिन्नक्रम IS A</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>इंन्द्र</t>
+          <t>तन्त्रयुक्ति</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>सहस्राक्ष</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>प्रजापति</t>
+          <t>BOTH</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>तन्त्रगुण</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2020,32 +2020,32 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>भिन्नक्रम IS A</t>
+          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>तन्त्रयुक्ति</t>
+          <t>अध्यायन</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>अध्यापन</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>BOTH</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>तन्त्रगुण</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2062,32 +2062,32 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
+          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>अध्यायन</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>अध्यापन</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>36</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2104,32 +2104,32 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
+          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>एकदोषज</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>त्रिदोषज</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>वातज</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2146,32 +2146,32 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
+          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>एकदोषज</t>
+          <t>अष्टांग हृदय</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>त्रिदोषज</t>
+          <t>सुश्रुत संहिता</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>वातज</t>
+          <t>अष्टांग संग्रह</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2188,32 +2188,32 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
+          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>अष्टांग हृदय</t>
+          <t>पिप्पलि</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>अपमार्ग</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>सुश्रुत संहिता</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>अष्टांग संग्रह</t>
+          <t>नीलिनी</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2230,32 +2230,32 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
+          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>पिप्पलि</t>
+          <t>वसन्त</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>अपमार्ग</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>शरत्</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>नीलिनी</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2272,32 +2272,32 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
+          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>वसन्त</t>
+          <t>NORTH</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>SOUTH</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>शरत्</t>
+          <t>EAST</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2314,32 +2314,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
+          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>NORTH</t>
+          <t>मधुर</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>SOUTH</t>
+          <t>आम्ल</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>EAST</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>तिक्त</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2356,32 +2356,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
+          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>मधुर</t>
+          <t>84</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>आम्ल</t>
+          <t>72</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>तिक्त</t>
+          <t>108</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2398,32 +2398,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
+          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>COPPERISH</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2440,32 +2440,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
+          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BLUE</t>
+          <t>तिर्यक्दोष</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>COPPERISH</t>
+          <t>अनुपस्थितदोश</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>ऊर्ध्वदोष</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2482,32 +2482,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
+          <t>अवपीडक सर्पि IS GIVEN IN</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>तिर्यक्दोष</t>
+          <t>छर्दिवेगधारण</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>पुरिषवेगधारण</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>अनुपस्थितदोश</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>ऊर्ध्वदोष</t>
+          <t>अश्रुवेगधारण</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2524,32 +2524,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>अवपीडक सर्पि IS GIVEN IN</t>
+          <t>WHICH IS RIGHT</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>छर्दिवेगधारण</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>पुरिषवेगधारण</t>
+          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>अश्रुवेगधारण</t>
+          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2566,32 +2566,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>WHICH IS RIGHT</t>
+          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
+          <t>ABUNDANT AVAILABILIT</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
+          <t>SHOULD HAVE MORE PARTS</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
+          <t>MULTIPLE COLORS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2608,32 +2608,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
+          <t>सुरा IS IDEAL अनुपान FOR</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>स्थूल</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ABUNDANT AVAILABILIT</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SHOULD HAVE MORE PARTS</t>
+          <t>शोष</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>MULTIPLE COLORS</t>
+          <t>विष</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2650,32 +2650,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>सुरा IS IDEAL अनुपान FOR</t>
+          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>स्थूल</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>कांस्य</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>शोष</t>
+          <t>स्वर्णा</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>विष</t>
+          <t>मुक्ता</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2692,32 +2692,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
+          <t>वात प्रकोप IS CAUSED BY</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>उष्ण युक्त रूक्ष</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>कांस्य</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>स्वर्णा</t>
+          <t>शीत युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>मुक्ता</t>
+          <t>उष्ण युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2734,32 +2734,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>वात प्रकोप IS CAUSED BY</t>
+          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>उष्ण युक्त रूक्ष</t>
+          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>शीत युक्त स्निग्ध</t>
+          <t>कर्ममिथ्यायोग</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>उष्ण युक्त स्निग्ध</t>
+          <t>वाक् मिथ्यायोग</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2776,32 +2776,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
+          <t>दूषिकI  IS मल OF</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
+          <t>कर्ण</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>नास</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>कर्ममिथ्यायोग</t>
+          <t>आस्य</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>वाक् मिथ्यायोग</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2813,292 +2813,250 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Samhita Adhyayana 2</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>दूषिकI  IS मल OF</t>
+          <t>Sushruta is known for?</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>कर्ण</t>
+          <t>Medicine</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>नास</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>आस्य</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>Toxicology</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Sushruta is father of surgery.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 2</t>
+          <t>Samhita Adhyayana 3</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Sushruta is known for?</t>
+          <t>Ashtanga Hridaya written by?</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>Charaka</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Sushruta</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Toxicology</t>
+          <t>Kashyapa</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Sushruta is father of surgery.</t>
+          <t>Vagbhata authored Ashtanga Hridaya.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 3</t>
+          <t>Sanskrit</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Ashtanga Hridaya written by?</t>
+          <t>Meaning of 'Vaidya'?</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Charaka</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Sushruta</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Kashyapa</t>
+          <t>King</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Vagbhata authored Ashtanga Hridaya.</t>
+          <t>Vaidya means physician.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Sanskrit</t>
+          <t>Shalakya Tantra</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Meaning of 'Vaidya'?</t>
+          <t>Shalakya deals with?</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Bones</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>Skin</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Vaidya means physician.</t>
+          <t>It deals with Urdhwajatrugata rogas.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Shalakya Tantra</t>
+          <t>Shalya Tantra</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Shalakya deals with?</t>
+          <t>Shalya Tantra deals with?</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Heart</t>
+          <t>Medicine</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Bones</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>It deals with Urdhwajatrugata rogas.</t>
+          <t>Shalya Tantra is surgical branch.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Shalya Tantra</t>
+          <t>Swasthavritta</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Shalya Tantra deals with?</t>
+          <t>Dinacharya refers to?</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Daily routine</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>Night routine</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Seasonal routine</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Daily routine</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
-        <is>
-          <t>Shalya Tantra is surgical branch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Swasthavritta</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Dinacharya refers to?</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Daily routine</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Night routine</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Seasonal routine</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>Daily routine</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
         <is>
           <t>Dinacharya means daily regimen.</t>
         </is>

</xml_diff>

<commit_message>
Started Student Performance dashboard backend
</commit_message>
<xml_diff>
--- a/AIAPGET_Questions.xlsx
+++ b/AIAPGET_Questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1679,168 +1679,168 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Parada is?</t>
+          <t>"UDAKADHARA" IS A LAYER OF SKIN ACCORDING TO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>CHARAKA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>SUSHRUTA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>LAGHU VAGBHATA</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>VRUDDHA VAGBHATA</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>CHARAKA</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Parada refers to mercury.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Research Methodology &amp; Statistics</t>
+          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Mean is?</t>
+          <t>Parada is?</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Median</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Mean is average.</t>
+          <t>Parada refers to mercury.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Roganidana</t>
+          <t>Research Methodology &amp; Statistics</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Nidana means?</t>
+          <t>Mean is?</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Treatment</t>
+          <t>Median</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Exercise</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Nidana refers to diagnosis.</t>
+          <t>Mean is average.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Roganidana</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Charaka Samhita belongs to?</t>
+          <t>Nidana means?</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Shalya</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>Treatment</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Shalakya</t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Kaumarabhritya</t>
+          <t>Exercise</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
+          <t>Nidana refers to diagnosis.</t>
         </is>
       </c>
     </row>
@@ -1852,37 +1852,37 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
+          <t>Charaka Samhita belongs to?</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>तैल</t>
+          <t>Shalya</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>वसा</t>
+          <t>Shalakya</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>मज्जा</t>
+          <t>Kaumarabhritya</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
         </is>
       </c>
     </row>
@@ -1894,32 +1894,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
+          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>शिशिर</t>
+          <t>तैल</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>वसा</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>मज्जा</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1936,32 +1936,32 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
+          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>शब्दकल्पद्रुम</t>
+          <t>शिशिर</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>तत्वचन्द्रिक</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>न्यायचन्द्रिक</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1978,32 +1978,32 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
+          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>चरक</t>
+          <t>शब्दकल्पद्रुम</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>तत्वचन्द्रिक</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>अग्निवेश</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>नागार्जुन</t>
+          <t>न्यायचन्द्रिक</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2020,32 +2020,32 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
+          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>इंन्द्र</t>
+          <t>चरक</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>सहस्राक्ष</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>प्रजापति</t>
+          <t>अग्निवेश</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>नागार्जुन</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2062,32 +2062,32 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>भिन्नक्रम IS A</t>
+          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>तन्त्रयुक्ति</t>
+          <t>इंन्द्र</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>सहस्राक्ष</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BOTH</t>
+          <t>प्रजापति</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>तन्त्रगुण</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2104,32 +2104,32 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
+          <t>भिन्नक्रम IS A</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>अध्यायन</t>
+          <t>तन्त्रयुक्ति</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>अध्यापन</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>BOTH</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>तन्त्रगुण</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2146,32 +2146,32 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
+          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>अध्यायन</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>अध्यापन</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2188,32 +2188,32 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
+          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>एकदोषज</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>त्रिदोषज</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>वातज</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>36</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2230,32 +2230,32 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
+          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>अष्टांग हृदय</t>
+          <t>एकदोषज</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>सुश्रुत संहिता</t>
+          <t>त्रिदोषज</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>अष्टांग संग्रह</t>
+          <t>वातज</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2272,32 +2272,32 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
+          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>पिप्पलि</t>
+          <t>अष्टांग हृदय</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>अपमार्ग</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>सुश्रुत संहिता</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>नीलिनी</t>
+          <t>अष्टांग संग्रह</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2314,32 +2314,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
+          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>वसन्त</t>
+          <t>पिप्पलि</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>अपमार्ग</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>शरत्</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>नीलिनी</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2356,32 +2356,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
+          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>NORTH</t>
+          <t>वसन्त</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>SOUTH</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>EAST</t>
+          <t>शरत्</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2398,32 +2398,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
+          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>मधुर</t>
+          <t>NORTH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>आम्ल</t>
+          <t>SOUTH</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>EAST</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>तिक्त</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2440,32 +2440,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
+          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>मधुर</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>आम्ल</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>तिक्त</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2482,32 +2482,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
+          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BLUE</t>
+          <t>84</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>72</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>COPPERISH</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>108</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2524,32 +2524,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
+          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>तिर्यक्दोष</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>अनुपस्थितदोश</t>
+          <t>COPPERISH</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>ऊर्ध्वदोष</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2566,32 +2566,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>अवपीडक सर्पि IS GIVEN IN</t>
+          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>छर्दिवेगधारण</t>
+          <t>तिर्यक्दोष</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>पुरिषवेगधारण</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>अनुपस्थितदोश</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>अश्रुवेगधारण</t>
+          <t>ऊर्ध्वदोष</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2608,32 +2608,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WHICH IS RIGHT</t>
+          <t>अवपीडक सर्पि IS GIVEN IN</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>छर्दिवेगधारण</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
+          <t>पुरिषवेगधारण</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
+          <t>अश्रुवेगधारण</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2650,32 +2650,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
+          <t>WHICH IS RIGHT</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ABUNDANT AVAILABILIT</t>
+          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SHOULD HAVE MORE PARTS</t>
+          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>MULTIPLE COLORS</t>
+          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2692,32 +2692,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>सुरा IS IDEAL अनुपान FOR</t>
+          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>स्थूल</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>ABUNDANT AVAILABILIT</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>शोष</t>
+          <t>SHOULD HAVE MORE PARTS</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>विष</t>
+          <t>MULTIPLE COLORS</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2734,32 +2734,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
+          <t>सुरा IS IDEAL अनुपान FOR</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>स्थूल</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>कांस्य</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>स्वर्णा</t>
+          <t>शोष</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>मुक्ता</t>
+          <t>विष</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2776,32 +2776,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>वात प्रकोप IS CAUSED BY</t>
+          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>उष्ण युक्त रूक्ष</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>कांस्य</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>शीत युक्त स्निग्ध</t>
+          <t>स्वर्णा</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>उष्ण युक्त स्निग्ध</t>
+          <t>मुक्ता</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2818,32 +2818,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
+          <t>वात प्रकोप IS CAUSED BY</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
+          <t>उष्ण युक्त रूक्ष</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>कर्ममिथ्यायोग</t>
+          <t>शीत युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>वाक् मिथ्यायोग</t>
+          <t>उष्ण युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2860,32 +2860,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>दूषिकI  IS मल OF</t>
+          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>कर्ण</t>
+          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>नास</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>आस्य</t>
+          <t>कर्ममिथ्यायोग</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>वाक् मिथ्यायोग</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2897,250 +2897,292 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 2</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Sushruta is known for?</t>
+          <t>दूषिकI  IS मल OF</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>कर्ण</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>नास</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>आस्य</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Toxicology</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Sushruta is father of surgery.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 3</t>
+          <t>Samhita Adhyayana 2</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ashtanga Hridaya written by?</t>
+          <t>Sushruta is known for?</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Charaka</t>
+          <t>Medicine</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Sushruta</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Kashyapa</t>
+          <t>Toxicology</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Vagbhata authored Ashtanga Hridaya.</t>
+          <t>Sushruta is father of surgery.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Sanskrit</t>
+          <t>Samhita Adhyayana 3</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Meaning of 'Vaidya'?</t>
+          <t>Ashtanga Hridaya written by?</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>Charaka</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>Sushruta</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>Kashyapa</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Vaidya means physician.</t>
+          <t>Vagbhata authored Ashtanga Hridaya.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Shalakya Tantra</t>
+          <t>Sanskrit</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Shalakya deals with?</t>
+          <t>Meaning of 'Vaidya'?</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Heart</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Bones</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>King</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>It deals with Urdhwajatrugata rogas.</t>
+          <t>Vaidya means physician.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Shalya Tantra</t>
+          <t>Shalakya Tantra</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Shalya Tantra deals with?</t>
+          <t>Shalakya deals with?</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Bones</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>Skin</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Shalya Tantra is surgical branch.</t>
+          <t>It deals with Urdhwajatrugata rogas.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>Shalya Tantra</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Shalya Tantra deals with?</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Pediatrics</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Diet</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Shalya Tantra is surgical branch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>Swasthavritta</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>Dinacharya refers to?</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>Daily routine</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>Night routine</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>Seasonal routine</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G66" t="inlineStr">
         <is>
           <t>Daily routine</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H66" t="inlineStr">
         <is>
           <t>Dinacharya means daily regimen.</t>
         </is>

</xml_diff>

<commit_message>
Refactor exam_db to use centralized database connection
</commit_message>
<xml_diff>
--- a/AIAPGET_Questions.xlsx
+++ b/AIAPGET_Questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1721,504 +1721,504 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Parada is?</t>
+          <t>Dwidhatvatmaka Purush includes</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Soumya and Agneya</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Shareera and Aatma</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Raja and Tama</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>Mahat and Aahankara</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Shareera and Aatma</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Parada refers to mercury.</t>
+          <t>PRESENT IN RACHANA BOOKS EXACT WORD NOT IN SAMHITAS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Research Methodology &amp; Statistics</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Mean is?</t>
+          <t>Total number of Jaala are</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Median</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>16</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Mean is average.</t>
+          <t>ACCORDING TO SUSHRUTA, VAGBHATA, BHAVAMISHRA, SHARANGADHARA. CHARAKA DIDN’T TOLD</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Roganidana</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nidana means?</t>
+          <t>Which of the following structures are involved in Akshepaka and Danda-Akshepaka?</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>ASTHI SANGHATA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Treatment</t>
+          <t>KURCHA</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>KANDARA</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Exercise</t>
+          <t>SEEMANTHA</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>KANDARA</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Nidana refers to diagnosis.</t>
+          <t>REFER SU.NI.1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Charaka Samhita belongs to?</t>
+          <t>Dhairya, Chyavana, Priti, Dehabala are said in the context of</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Shalya</t>
+          <t>Shuddha Aartava</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>Shuddha Shukra</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Shalakya</t>
+          <t>Shukra Functions</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Kaumarabhritya</t>
+          <t>Aartava Functions</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>Shukra Functions</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
+          <t>KNOW DIFFERENCE BETWEEN KARMA AND GUNA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
+          <t>Sira Vedhya in Dakodara is done 4 Angula left of</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>तैल</t>
+          <t>Kurcha</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>Sevani</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>वसा</t>
+          <t>Seemantha</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>मज्जा</t>
+          <t>Asthi sanghata</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>Sevani</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>REFER SU.SHA.8</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
+          <t>Maternal surface of the Placenta develops from</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>शिशिर</t>
+          <t>Decidua Basalis</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>Decidua Capsularis</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>Chorion Leavae</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>Chorion Frondosum</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>Decidua Basalis</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>MATERNAL COMPONENT ENTIRELY DEVOLOPS FROM THIS WHICH MAKES BASAL PLATE WHICH FACES UTERINE WALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
+          <t>Which of the following is a Sesamoid bone?</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>शब्दकल्पद्रुम</t>
+          <t>Palatine</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>तत्वचन्द्रिक</t>
+          <t>Mandible</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>Maxilla</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>न्यायचन्द्रिक</t>
+          <t>Patella</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>Patella</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>PATELLA IS THE LARGEST SESMOID BONE, WHICH DEVELOPS INSIDE THICK TENDON OF QUADRICEPS FEMORIS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
+          <t>Which of the following type of Snayu is present in Parshwa?</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>चरक</t>
+          <t>Prutu</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>Sushira</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>अग्निवेश</t>
+          <t>Pratanavati</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>नागार्जुन</t>
+          <t>Vrutta</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>Pratanavati</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>REFER SU. SHA.5</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
+          <t>Parada is?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>इंन्द्र</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>सहस्राक्ष</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>प्रजापति</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Parada refers to mercury.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>भिन्नक्रम IS A</t>
+          <t>Mitra panchaka varga dravyas used in which Bhasma pariksha</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>तन्त्रयुक्ति</t>
+          <t>Apunarbhava</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>Nirutta</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>BOTH</t>
+          <t>Varitara</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>तन्त्रगुण</t>
+          <t>Rekhapurna</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>Apunarbhava</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>APUNARBHAVA IS A HIGH TEMPERATURE METALLURGICAL REDUCTION TEST BY USING ORGANIC COMPUNDS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Research Methodology &amp; Statistics</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
+          <t>Mean is?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>अध्यायन</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>अध्यापन</t>
+          <t>Median</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Mean is average.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Roganidana</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
+          <t>Nidana means?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>Treatment</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>Exercise</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Nidana refers to diagnosis.</t>
         </is>
       </c>
     </row>
@@ -2230,37 +2230,37 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
+          <t>Charaka Samhita belongs to?</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>एकदोषज</t>
+          <t>Shalya</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>त्रिदोषज</t>
+          <t>Shalakya</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>वातज</t>
+          <t>Kaumarabhritya</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
         </is>
       </c>
     </row>
@@ -2272,32 +2272,32 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
+          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>अष्टांग हृदय</t>
+          <t>तैल</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>सुश्रुत संहिता</t>
+          <t>वसा</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>अष्टांग संग्रह</t>
+          <t>मज्जा</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2314,32 +2314,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
+          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>पिप्पलि</t>
+          <t>शिशिर</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>अपमार्ग</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>नीलिनी</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2356,32 +2356,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
+          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>वसन्त</t>
+          <t>शब्दकल्पद्रुम</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>तत्वचन्द्रिक</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>शरत्</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>न्यायचन्द्रिक</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2398,32 +2398,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
+          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NORTH</t>
+          <t>चरक</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>SOUTH</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>EAST</t>
+          <t>अग्निवेश</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>नागार्जुन</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2440,32 +2440,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
+          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>मधुर</t>
+          <t>इंन्द्र</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>आम्ल</t>
+          <t>सहस्राक्ष</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>प्रजापति</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>तिक्त</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2482,32 +2482,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
+          <t>भिन्नक्रम IS A</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>तन्त्रयुक्ति</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>BOTH</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>तन्त्रगुण</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2524,32 +2524,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
+          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>BLUE</t>
+          <t>अध्यायन</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>अध्यापन</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>COPPERISH</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2566,32 +2566,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
+          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>तिर्यक्दोष</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>अनुपस्थितदोश</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>ऊर्ध्वदोष</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>36</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2608,32 +2608,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>अवपीडक सर्पि IS GIVEN IN</t>
+          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>छर्दिवेगधारण</t>
+          <t>एकदोषज</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>पुरिषवेगधारण</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>त्रिदोषज</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>अश्रुवेगधारण</t>
+          <t>वातज</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2650,32 +2650,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WHICH IS RIGHT</t>
+          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>अष्टांग हृदय</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
+          <t>सुश्रुत संहिता</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
+          <t>अष्टांग संग्रह</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2692,32 +2692,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
+          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>पिप्पलि</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ABUNDANT AVAILABILIT</t>
+          <t>अपमार्ग</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SHOULD HAVE MORE PARTS</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>MULTIPLE COLORS</t>
+          <t>नीलिनी</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2734,32 +2734,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>सुरा IS IDEAL अनुपान FOR</t>
+          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>स्थूल</t>
+          <t>वसन्त</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>शोष</t>
+          <t>शरत्</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>विष</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2776,32 +2776,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
+          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>NORTH</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>कांस्य</t>
+          <t>SOUTH</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>स्वर्णा</t>
+          <t>EAST</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>मुक्ता</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2818,32 +2818,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>वात प्रकोप IS CAUSED BY</t>
+          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>उष्ण युक्त रूक्ष</t>
+          <t>मधुर</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>आम्ल</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>शीत युक्त स्निग्ध</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>उष्ण युक्त स्निग्ध</t>
+          <t>तिक्त</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2860,32 +2860,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
+          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
+          <t>84</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>72</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>कर्ममिथ्यायोग</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>वाक् मिथ्यायोग</t>
+          <t>108</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2902,32 +2902,32 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>दूषिकI  IS मल OF</t>
+          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>कर्ण</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>नास</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>आस्य</t>
+          <t>COPPERISH</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2939,250 +2939,628 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 2</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Sushruta is known for?</t>
+          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>तिर्यक्दोष</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>अनुपस्थितदोश</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Toxicology</t>
+          <t>ऊर्ध्वदोष</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Sushruta is father of surgery.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 3</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ashtanga Hridaya written by?</t>
+          <t>अवपीडक सर्पि IS GIVEN IN</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Charaka</t>
+          <t>छर्दिवेगधारण</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Sushruta</t>
+          <t>पुरिषवेगधारण</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Kashyapa</t>
+          <t>अश्रुवेगधारण</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Vagbhata authored Ashtanga Hridaya.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Sanskrit</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Meaning of 'Vaidya'?</t>
+          <t>WHICH IS RIGHT</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Vaidya means physician.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Shalakya Tantra</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Shalakya deals with?</t>
+          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Heart</t>
+          <t>ABUNDANT AVAILABILIT</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Bones</t>
+          <t>SHOULD HAVE MORE PARTS</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>MULTIPLE COLORS</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>It deals with Urdhwajatrugata rogas.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Shalya Tantra</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Shalya Tantra deals with?</t>
+          <t>सुरा IS IDEAL अनुपान FOR</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>स्थूल</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>शोष</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>विष</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Shalya Tantra is surgical branch.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>Samhita Adhyayana 1</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>रजत</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>कांस्य</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>स्वर्णा</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>मुक्ता</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>रजत</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>REFER BOOK</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Samhita Adhyayana 1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>वात प्रकोप IS CAUSED BY</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>उष्ण युक्त रूक्ष</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>शीत युक्त रूक्ष</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>शीत युक्त स्निग्ध</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>उष्ण युक्त स्निग्ध</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>शीत युक्त रूक्ष</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>REFER BOOK</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Samhita Adhyayana 1</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>कर्ममिथ्यायोग</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>वाक् मिथ्यायोग</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>REFER BOOK</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Samhita Adhyayana 1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>दूषिकI  IS मल OF</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>कर्ण</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>नास</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>आस्य</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>नेत्र</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>नेत्र</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>REFER BOOK</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Samhita Adhyayana 2</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Sushruta is known for?</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Pediatrics</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Toxicology</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Sushruta is father of surgery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Samhita Adhyayana 3</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Ashtanga Hridaya written by?</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Charaka</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Sushruta</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Vagbhata</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Kashyapa</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Vagbhata</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Vagbhata authored Ashtanga Hridaya.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Sanskrit</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Meaning of 'Vaidya'?</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Doctor</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Teacher</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>King</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Doctor</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Vaidya means physician.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Shalakya Tantra</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Shalakya deals with?</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ENT &amp; Eye</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Heart</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Bones</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Skin</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>ENT &amp; Eye</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>It deals with Urdhwajatrugata rogas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Shalya Tantra</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Shalya Tantra deals with?</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Pediatrics</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Diet</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Shalya Tantra is surgical branch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
           <t>Swasthavritta</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>Dinacharya refers to?</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>Daily routine</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>Night routine</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>Seasonal routine</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G75" t="inlineStr">
         <is>
           <t>Daily routine</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H75" t="inlineStr">
         <is>
           <t>Dinacharya means daily regimen.</t>
         </is>

</xml_diff>

<commit_message>
Migrate AIAPGET CBT from SQLite to PostgreSQL
</commit_message>
<xml_diff>
--- a/AIAPGET_Questions.xlsx
+++ b/AIAPGET_Questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,42 +587,42 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kaumarabhritya</t>
+          <t>Dravyaguna</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kaumarabhritya deals with?</t>
+          <t>What is the currently accepted botanical name for the Ayurvedic herb Tagara?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Children</t>
+          <t>Valeriana officinalis</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Adults</t>
+          <t>Valeriana jatamansi</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Elderly</t>
+          <t>Valeriana hardwickii</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Nardostachys jatamansi</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Children</t>
+          <t>Valeriana jatamansi</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>It is pediatrics.</t>
+          <t>While historically known as Valeriana wallichii, modern botanical taxonomy recognizes Valeriana jatamansi Jones as the accepted name. Valeriana officinalis is European Valerian, and Nardostachys jatamansi is a completely different plant (Jatamansi/Spikenard).</t>
         </is>
       </c>
     </row>
@@ -634,205 +634,205 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>kaumarabhritya is also called as</t>
+          <t>Kaumarabhritya deals with?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>bala roga</t>
+          <t>Children</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>kumara vijnana</t>
+          <t>Adults</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>kumara stree vijnana</t>
+          <t>Elderly</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>Women</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>bala roga</t>
+          <t>Children</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>refer book</t>
+          <t>It is pediatrics.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>Kaumarabhritya</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vata is composed of?</t>
+          <t>kaumarabhritya is also called as</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Agni</t>
+          <t>bala roga</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Vayu + Akasha</t>
+          <t>kumara vijnana</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Jala</t>
+          <t>kumara stree vijnana</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Prithvi</t>
+          <t>all</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Vayu + Akasha</t>
+          <t>bala roga</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Vata is formed by Vayu and Akasha.</t>
+          <t>refer book</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kriya Sharira</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pitta is mainly responsible for?</t>
+          <t>Vata is composed of?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Movement</t>
+          <t>Agni</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Digestion</t>
+          <t>Vayu + Akasha</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Jala</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Lubrication</t>
+          <t>Prithvi</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Digestion</t>
+          <t>Vayu + Akasha</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Pitta governs digestion and metabolism.</t>
+          <t>Vata is formed by Vayu and Akasha.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Modern Topics</t>
+          <t>Kriya Sharira</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>WHO stands for?</t>
+          <t>Pitta is mainly responsible for?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>World Health Organization</t>
+          <t>Movement</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>World Human Org</t>
+          <t>Digestion</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Health World Org</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Lubrication</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>World Health Organization</t>
+          <t>Digestion</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>WHO is global health body.</t>
+          <t>Pitta governs digestion and metabolism.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Modern Topics</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>विवर्त वाद IS ACCEPTE BY</t>
+          <t>WHO stands for?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>World Health Organization</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>World Human Org</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>चार्वाक</t>
+          <t>Health World Org</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>World Health Organization</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>WHO is global health body.</t>
         </is>
       </c>
     </row>
@@ -844,32 +844,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IN सृष्टि उत्पत्ति, नप्रकृति न विकृति IS</t>
+          <t>विवर्त वाद IS ACCEPTE BY</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>अहंकार</t>
+          <t>जैन</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>वैशेषिक</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>महत्</t>
+          <t>चार्वाक</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>मनस्</t>
+          <t>वेदान्त</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>वेदान्त</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -886,32 +886,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ACCORDING TO कारिकावलि, THE सामान्य WHICH PERVADES ALL द्रव्य, गुण , कर्म IS CALLED AS</t>
+          <t>IN सृष्टि उत्पत्ति, नप्रकृति न विकृति IS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>परसामान्य</t>
+          <t>अहंकार</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>अपरसामान्य</t>
+          <t>पुरुष</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">परापरसामान्य </t>
+          <t>महत्</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>विशेषसामन्य</t>
+          <t>मनस्</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>परसामान्य</t>
+          <t>पुरुष</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -928,32 +928,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>THE अभाव WHICH IS BOTH  आदि AND अनन्त IS</t>
+          <t>ACCORDING TO कारिकावलि, THE सामान्य WHICH PERVADES ALL द्रव्य, गुण , कर्म IS CALLED AS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>प्राग्भाव</t>
+          <t>परसामान्य</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>प्रध्वंसाभाव</t>
+          <t>अपरसामान्य</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>अन्योन्याभाव</t>
+          <t xml:space="preserve">परापरसामान्य </t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>सर्वाभाव</t>
+          <t>विशेषसामन्य</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>अन्योन्याभाव</t>
+          <t>परसामान्य</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -970,32 +970,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IN अनुमान, परामर्श WILL EVOLVE</t>
+          <t>THE अभाव WHICH IS BOTH  आदि AND अनन्त IS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AFTER ESTABLISHMENT OF व्याप्ति</t>
+          <t>प्राग्भाव</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BEFORE व्याप्ति</t>
+          <t>प्रध्वंसाभाव</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>AFTER पक्षधर्मत</t>
+          <t>अन्योन्याभाव</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>सर्वाभाव</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>AFTER पक्षधर्मत</t>
+          <t>अन्योन्याभाव</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1012,32 +1012,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>THE STATEMENT, पृथ्वि IS DIFFERENT FROM OTHER भूतs BECAUSE THEY DONT HAVE गन्धगुण IS AN EXAMPLE OF</t>
+          <t>IN अनुमान, परामर्श WILL EVOLVE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>केवलान्वयि</t>
+          <t>AFTER ESTABLISHMENT OF व्याप्ति</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>केवलव्यतिरेकि</t>
+          <t>BEFORE व्याप्ति</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOTH </t>
+          <t>AFTER पक्षधर्मत</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>विशेष व्यतिरेकि</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>केवलव्यतिरेकि</t>
+          <t>AFTER पक्षधर्मत</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1054,32 +1054,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>धर्म, अधर्म ARE पदार्थ/DRAVYA ACCORDING TO</t>
+          <t>THE STATEMENT, पृथ्वि IS DIFFERENT FROM OTHER भूतs BECAUSE THEY DONT HAVE गन्धगुण IS AN EXAMPLE OF</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>सांख्य</t>
+          <t>केवलान्वयि</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>केवलव्यतिरेकि</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t xml:space="preserve">BOTH </t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>बौद्ध</t>
+          <t>विशेष व्यतिरेकि</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>केवलव्यतिरेकि</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1096,32 +1096,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>विशिष्टाद्वैत POPULARISED BY</t>
+          <t>धर्म, अधर्म ARE पदार्थ/DRAVYA ACCORDING TO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>रामानुजाचार्य</t>
+          <t>सांख्य</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>शंकराचार्य</t>
+          <t>जैन</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>मध्वाचार्य</t>
+          <t>वेदान्त</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>प्रभाकर</t>
+          <t>बौद्ध</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>रामानुजाचार्य</t>
+          <t>जैन</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1138,32 +1138,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>चेष्टा प्रमाण IS ACCEPTED BY</t>
+          <t>विशिष्टाद्वैत POPULARISED BY</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>प्रभाकर मीमांस</t>
+          <t>रामानुजाचार्य</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>पौराणिक</t>
+          <t>शंकराचार्य</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>तान्त्रिक</t>
+          <t>मध्वाचार्य</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>मध्व</t>
+          <t>प्रभाकर</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>तान्त्रिक</t>
+          <t>रामानुजाचार्य</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1180,32 +1180,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FROM WHICH दर्शन AYURVEDA TAKEN षट् पदार्थ</t>
+          <t>चेष्टा प्रमाण IS ACCEPTED BY</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">सांख्य </t>
+          <t>प्रभाकर मीमांस</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>योग</t>
+          <t>पौराणिक</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>न्याय</t>
+          <t>तान्त्रिक</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>मध्व</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>तान्त्रिक</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1222,32 +1222,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ACCORDING TO चरक अतिवाहिक पुरुष IS NOT ASSOCIATED WITH</t>
+          <t>FROM WHICH दर्शन AYURVEDA TAKEN षट् पदार्थ</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>मन</t>
+          <t xml:space="preserve">सांख्य </t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">मन- आकाश       </t>
+          <t>योग</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>इन्द्रिय</t>
+          <t>न्याय</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>वैशेषिक</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>इन्द्रिय</t>
+          <t>वैशेषिक</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1264,32 +1264,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>षट् पदार्थ ARE CALLED BY चरक AS</t>
+          <t>ACCORDING TO चरक अतिवाहिक पुरुष IS NOT ASSOCIATED WITH</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>कार्य</t>
+          <t>मन</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>पदार्थ</t>
+          <t xml:space="preserve">मन- आकाश       </t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>इन्द्रिय</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>विशेष</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>इन्द्रिय</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1306,32 +1306,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>WHICH इन्द्रिय प्रत्यक्ष प्रमाण NOT USED TO EXAMINE रोगि</t>
+          <t>षट् पदार्थ ARE CALLED BY चरक AS</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>स्पर्शनेन्द्रिय</t>
+          <t>कार्य</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">चक्षुरेन्द्रिय </t>
+          <t>पदार्थ</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>रस्नेन्द्रिय</t>
+          <t>कारण</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>घ्राणेन्द्रिय</t>
+          <t>विशेष</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>रस्नेन्द्रिय</t>
+          <t>कारण</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1348,32 +1348,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>यस्य विवरणे शक्ति: IS</t>
+          <t>WHICH इन्द्रिय प्रत्यक्ष प्रमाण NOT USED TO EXAMINE रोगि</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>खर</t>
+          <t>स्पर्शनेन्द्रिय</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">द्रव </t>
+          <t xml:space="preserve">चक्षुरेन्द्रिय </t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">सूक्ष्म       </t>
+          <t>रस्नेन्द्रिय</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>घ्राणेन्द्रिय</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>सूक्ष्म</t>
+          <t>रस्नेन्द्रिय</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1390,32 +1390,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>THE ELASTICITY OF RUBBER IS AN EXAMPLE FOR</t>
+          <t>यस्य विवरणे शक्ति: IS</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">वेगाख्य संस्कार </t>
+          <t>खर</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>स्थितिस्थापक</t>
+          <t xml:space="preserve">द्रव </t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>प्रतिविरुद्ध</t>
+          <t xml:space="preserve">सूक्ष्म       </t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>भावनाख्य संस्कार</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>स्थितिस्थापक</t>
+          <t>सूक्ष्म</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1432,32 +1432,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FOLLOWING IS NOT THE USE OF काल</t>
+          <t>THE ELASTICITY OF RUBBER IS AN EXAMPLE FOR</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DRUG ADMINISTRATION</t>
+          <t xml:space="preserve">वेगाख्य संस्कार </t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KNOWING DISESE STATUS</t>
+          <t>स्थितिस्थापक</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">KNOWING SEASONS      </t>
+          <t>प्रतिविरुद्ध</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>भावनाख्य संस्कार</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>स्थितिस्थापक</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1474,32 +1474,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>अविनावभाव सम्बन्ध IS</t>
+          <t>FOLLOWING IS NOT THE USE OF काल</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>सामान्यतो दॄष्ट अनुमान</t>
+          <t>DRUG ADMINISTRATION</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>अन्वयव्यतिरेकि</t>
+          <t>KNOWING DISESE STATUS</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>कल्पना</t>
+          <t xml:space="preserve">KNOWING SEASONS      </t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>व्याप्ति</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>व्याप्ति</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1516,163 +1516,163 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SEE THE IMAGE AND IDENTIFY THE अभाव</t>
+          <t>अविनावभाव सम्बन्ध IS</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>प्राग्भाव</t>
+          <t>सामान्यतो दॄष्ट अनुमान</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>अत्यंतअभाव</t>
+          <t>अन्वयव्यतिरेकि</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>प्रध्वंसाभाव</t>
+          <t>कल्पना</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>व्याप्ति</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>प्रध्वंसाभाव</t>
+          <t>व्याप्ति</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>SEE BOOK</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Panchakarma</t>
+          <t>Padartha VIjnana</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Vamana is?</t>
+          <t>SEE THE IMAGE AND IDENTIFY THE अभाव</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Emesis</t>
+          <t>प्राग्भाव</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Purgation</t>
+          <t>अत्यंतअभाव</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Enema</t>
+          <t>प्रध्वंसाभाव</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Nasal therapy</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Emesis</t>
+          <t>प्रध्वंसाभाव</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Vamana is therapeutic emesis.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Prasooti Tantra &amp; Stree Roga</t>
+          <t>Panchakarma</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Garbhini means?</t>
+          <t>Vamana is?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Pregnant woman</t>
+          <t>Emesis</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Child</t>
+          <t>Purgation</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>Enema</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Nurse</t>
+          <t>Nasal therapy</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Pregnant woman</t>
+          <t>Emesis</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Garbhini refers to pregnant woman.</t>
+          <t>Vamana is therapeutic emesis.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rachana Sharira</t>
+          <t>Prasooti Tantra &amp; Stree Roga</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Number of bones in adult human body?</t>
+          <t>Garbhini means?</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>Pregnant woman</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>Child</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>Nurse</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>Pregnant woman</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Adult human body has 206 bones.</t>
+          <t>Garbhini refers to pregnant woman.</t>
         </is>
       </c>
     </row>
@@ -1684,37 +1684,37 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>"UDAKADHARA" IS A LAYER OF SKIN ACCORDING TO</t>
+          <t>Number of bones in adult human body?</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CHARAKA</t>
+          <t>206</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>SUSHRUTA</t>
+          <t>210</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LAGHU VAGBHATA</t>
+          <t>300</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>VRUDDHA VAGBHATA</t>
+          <t>180</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>CHARAKA</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Adult human body has 206 bones.</t>
         </is>
       </c>
     </row>
@@ -1726,37 +1726,37 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dwidhatvatmaka Purush includes</t>
+          <t>"UDAKADHARA" IS A LAYER OF SKIN ACCORDING TO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Soumya and Agneya</t>
+          <t>CHARAKA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Shareera and Aatma</t>
+          <t>SUSHRUTA</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Raja and Tama</t>
+          <t>LAGHU VAGBHATA</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Mahat and Aahankara</t>
+          <t>VRUDDHA VAGBHATA</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Shareera and Aatma</t>
+          <t>CHARAKA</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>PRESENT IN RACHANA BOOKS EXACT WORD NOT IN SAMHITAS</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
@@ -1768,37 +1768,37 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Total number of Jaala are</t>
+          <t>Dwidhatvatmaka Purush includes</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>Soumya and Agneya</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>Shareera and Aatma</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>Raja and Tama</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>Mahat and Aahankara</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>Shareera and Aatma</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>ACCORDING TO SUSHRUTA, VAGBHATA, BHAVAMISHRA, SHARANGADHARA. CHARAKA DIDN’T TOLD</t>
+          <t>PRESENT IN RACHANA BOOKS EXACT WORD NOT IN SAMHITAS</t>
         </is>
       </c>
     </row>
@@ -1810,37 +1810,37 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Which of the following structures are involved in Akshepaka and Danda-Akshepaka?</t>
+          <t>Total number of Jaala are</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ASTHI SANGHATA</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>KURCHA</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>KANDARA</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>SEEMANTHA</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KANDARA</t>
+          <t>16</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>REFER SU.NI.1</t>
+          <t>ACCORDING TO SUSHRUTA, VAGBHATA, BHAVAMISHRA, SHARANGADHARA. CHARAKA DIDN’T TOLD</t>
         </is>
       </c>
     </row>
@@ -1852,37 +1852,37 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dhairya, Chyavana, Priti, Dehabala are said in the context of</t>
+          <t>Which of the following structures are involved in Akshepaka and Danda-Akshepaka?</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Shuddha Aartava</t>
+          <t>ASTHI SANGHATA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Shuddha Shukra</t>
+          <t>KURCHA</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Shukra Functions</t>
+          <t>KANDARA</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Aartava Functions</t>
+          <t>SEEMANTHA</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Shukra Functions</t>
+          <t>KANDARA</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>KNOW DIFFERENCE BETWEEN KARMA AND GUNA</t>
+          <t>REFER SU.NI.1</t>
         </is>
       </c>
     </row>
@@ -1894,37 +1894,37 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Sira Vedhya in Dakodara is done 4 Angula left of</t>
+          <t>Dhairya, Chyavana, Priti, Dehabala are said in the context of</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Kurcha</t>
+          <t>Shuddha Aartava</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Sevani</t>
+          <t>Shuddha Shukra</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Seemantha</t>
+          <t>Shukra Functions</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Asthi sanghata</t>
+          <t>Aartava Functions</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Sevani</t>
+          <t>Shukra Functions</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>REFER SU.SHA.8</t>
+          <t>KNOW DIFFERENCE BETWEEN KARMA AND GUNA</t>
         </is>
       </c>
     </row>
@@ -1936,37 +1936,37 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Maternal surface of the Placenta develops from</t>
+          <t>Sira Vedhya in Dakodara is done 4 Angula left of</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Decidua Basalis</t>
+          <t>Kurcha</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Decidua Capsularis</t>
+          <t>Sevani</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Chorion Leavae</t>
+          <t>Seemantha</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Chorion Frondosum</t>
+          <t>Asthi sanghata</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Decidua Basalis</t>
+          <t>Sevani</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>MATERNAL COMPONENT ENTIRELY DEVOLOPS FROM THIS WHICH MAKES BASAL PLATE WHICH FACES UTERINE WALL</t>
+          <t>REFER SU.SHA.8</t>
         </is>
       </c>
     </row>
@@ -1978,37 +1978,37 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Which of the following is a Sesamoid bone?</t>
+          <t>Maternal surface of the Placenta develops from</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Palatine</t>
+          <t>Decidua Basalis</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Mandible</t>
+          <t>Decidua Capsularis</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Maxilla</t>
+          <t>Chorion Leavae</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Patella</t>
+          <t>Chorion Frondosum</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Patella</t>
+          <t>Decidua Basalis</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>PATELLA IS THE LARGEST SESMOID BONE, WHICH DEVELOPS INSIDE THICK TENDON OF QUADRICEPS FEMORIS</t>
+          <t>MATERNAL COMPONENT ENTIRELY DEVOLOPS FROM THIS WHICH MAKES BASAL PLATE WHICH FACES UTERINE WALL</t>
         </is>
       </c>
     </row>
@@ -2020,79 +2020,79 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Which of the following type of Snayu is present in Parshwa?</t>
+          <t>Which of the following is a Sesamoid bone?</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Prutu</t>
+          <t>Palatine</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Sushira</t>
+          <t>Mandible</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Pratanavati</t>
+          <t>Maxilla</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Vrutta</t>
+          <t>Patella</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Pratanavati</t>
+          <t>Patella</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>REFER SU. SHA.5</t>
+          <t>PATELLA IS THE LARGEST SESMOID BONE, WHICH DEVELOPS INSIDE THICK TENDON OF QUADRICEPS FEMORIS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Parada is?</t>
+          <t>Which of the following type of Snayu is present in Parshwa?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Prutu</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Sushira</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Pratanavati</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>Vrutta</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Pratanavati</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Parada refers to mercury.</t>
+          <t>REFER SU. SHA.5</t>
         </is>
       </c>
     </row>
@@ -2104,163 +2104,163 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Mitra panchaka varga dravyas used in which Bhasma pariksha</t>
+          <t>Parada is?</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Apunarbhava</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Nirutta</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Varitara</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Rekhapurna</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Apunarbhava</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>APUNARBHAVA IS A HIGH TEMPERATURE METALLURGICAL REDUCTION TEST BY USING ORGANIC COMPUNDS</t>
+          <t>Parada refers to mercury.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Research Methodology &amp; Statistics</t>
+          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mean is?</t>
+          <t>Mitra panchaka varga dravyas used in which Bhasma pariksha</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Apunarbhava</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Median</t>
+          <t>Nirutta</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>Varitara</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Rekhapurna</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Apunarbhava</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Mean is average.</t>
+          <t>APUNARBHAVA IS A HIGH TEMPERATURE METALLURGICAL REDUCTION TEST BY USING ORGANIC COMPUNDS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Roganidana</t>
+          <t>Research Methodology &amp; Statistics</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Nidana means?</t>
+          <t>Mean is?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Treatment</t>
+          <t>Median</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Exercise</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Nidana refers to diagnosis.</t>
+          <t>Mean is average.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Roganidana</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Charaka Samhita belongs to?</t>
+          <t>Nidana means?</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Shalya</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>Treatment</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Shalakya</t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Kaumarabhritya</t>
+          <t>Exercise</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
+          <t>Nidana refers to diagnosis.</t>
         </is>
       </c>
     </row>
@@ -2272,37 +2272,37 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
+          <t>Charaka Samhita belongs to?</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>तैल</t>
+          <t>Shalya</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>वसा</t>
+          <t>Shalakya</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>मज्जा</t>
+          <t>Kaumarabhritya</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
         </is>
       </c>
     </row>
@@ -2314,32 +2314,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
+          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>शिशिर</t>
+          <t>तैल</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>वसा</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>मज्जा</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2356,32 +2356,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
+          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>शब्दकल्पद्रुम</t>
+          <t>शिशिर</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>तत्वचन्द्रिक</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>न्यायचन्द्रिक</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2398,32 +2398,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
+          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>चरक</t>
+          <t>शब्दकल्पद्रुम</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>तत्वचन्द्रिक</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>अग्निवेश</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>नागार्जुन</t>
+          <t>न्यायचन्द्रिक</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2440,32 +2440,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
+          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>इंन्द्र</t>
+          <t>चरक</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>सहस्राक्ष</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>प्रजापति</t>
+          <t>अग्निवेश</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>नागार्जुन</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2482,32 +2482,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>भिन्नक्रम IS A</t>
+          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>तन्त्रयुक्ति</t>
+          <t>इंन्द्र</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>सहस्राक्ष</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>BOTH</t>
+          <t>प्रजापति</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>तन्त्रगुण</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2524,32 +2524,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
+          <t>भिन्नक्रम IS A</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>अध्यायन</t>
+          <t>तन्त्रयुक्ति</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>अध्यापन</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>BOTH</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>तन्त्रगुण</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2566,32 +2566,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
+          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>अध्यायन</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>अध्यापन</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2608,32 +2608,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
+          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>एकदोषज</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>त्रिदोषज</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>वातज</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>36</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2650,32 +2650,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
+          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>अष्टांग हृदय</t>
+          <t>एकदोषज</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>सुश्रुत संहिता</t>
+          <t>त्रिदोषज</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>अष्टांग संग्रह</t>
+          <t>वातज</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2692,32 +2692,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
+          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>पिप्पलि</t>
+          <t>अष्टांग हृदय</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>अपमार्ग</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>सुश्रुत संहिता</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>नीलिनी</t>
+          <t>अष्टांग संग्रह</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2734,32 +2734,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
+          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>वसन्त</t>
+          <t>पिप्पलि</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>अपमार्ग</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>शरत्</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>नीलिनी</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2776,32 +2776,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
+          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>NORTH</t>
+          <t>वसन्त</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>SOUTH</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>EAST</t>
+          <t>शरत्</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2818,32 +2818,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
+          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>मधुर</t>
+          <t>NORTH</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>आम्ल</t>
+          <t>SOUTH</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>EAST</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>तिक्त</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2860,32 +2860,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
+          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>मधुर</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>आम्ल</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>तिक्त</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2902,32 +2902,32 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
+          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>BLUE</t>
+          <t>84</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>72</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>COPPERISH</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>108</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2944,32 +2944,32 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
+          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>तिर्यक्दोष</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>अनुपस्थितदोश</t>
+          <t>COPPERISH</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>ऊर्ध्वदोष</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2986,32 +2986,32 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>अवपीडक सर्पि IS GIVEN IN</t>
+          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>छर्दिवेगधारण</t>
+          <t>तिर्यक्दोष</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>पुरिषवेगधारण</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>अनुपस्थितदोश</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>अश्रुवेगधारण</t>
+          <t>ऊर्ध्वदोष</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3028,32 +3028,32 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>WHICH IS RIGHT</t>
+          <t>अवपीडक सर्पि IS GIVEN IN</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>छर्दिवेगधारण</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
+          <t>पुरिषवेगधारण</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
+          <t>अश्रुवेगधारण</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3070,32 +3070,32 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
+          <t>WHICH IS RIGHT</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>ABUNDANT AVAILABILIT</t>
+          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>SHOULD HAVE MORE PARTS</t>
+          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>MULTIPLE COLORS</t>
+          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3112,32 +3112,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>सुरा IS IDEAL अनुपान FOR</t>
+          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>स्थूल</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>ABUNDANT AVAILABILIT</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>शोष</t>
+          <t>SHOULD HAVE MORE PARTS</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>विष</t>
+          <t>MULTIPLE COLORS</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3154,32 +3154,32 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
+          <t>सुरा IS IDEAL अनुपान FOR</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>स्थूल</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>कांस्य</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>स्वर्णा</t>
+          <t>शोष</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>मुक्ता</t>
+          <t>विष</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3196,32 +3196,32 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>वात प्रकोप IS CAUSED BY</t>
+          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>उष्ण युक्त रूक्ष</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>कांस्य</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>शीत युक्त स्निग्ध</t>
+          <t>स्वर्णा</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>उष्ण युक्त स्निग्ध</t>
+          <t>मुक्ता</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3238,32 +3238,32 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
+          <t>वात प्रकोप IS CAUSED BY</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
+          <t>उष्ण युक्त रूक्ष</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>कर्ममिथ्यायोग</t>
+          <t>शीत युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>वाक् मिथ्यायोग</t>
+          <t>उष्ण युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3280,32 +3280,32 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>दूषिकI  IS मल OF</t>
+          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>कर्ण</t>
+          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>नास</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>आस्य</t>
+          <t>कर्ममिथ्यायोग</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>वाक् मिथ्यायोग</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3317,250 +3317,292 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 2</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Sushruta is known for?</t>
+          <t>दूषिकI  IS मल OF</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>कर्ण</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>नास</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>आस्य</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Toxicology</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Sushruta is father of surgery.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 3</t>
+          <t>Samhita Adhyayana 2</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Ashtanga Hridaya written by?</t>
+          <t>Sushruta is known for?</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Charaka</t>
+          <t>Medicine</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Sushruta</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Kashyapa</t>
+          <t>Toxicology</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Vagbhata authored Ashtanga Hridaya.</t>
+          <t>Sushruta is father of surgery.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Sanskrit</t>
+          <t>Samhita Adhyayana 3</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Meaning of 'Vaidya'?</t>
+          <t>Ashtanga Hridaya written by?</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>Charaka</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>Sushruta</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>Kashyapa</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Vaidya means physician.</t>
+          <t>Vagbhata authored Ashtanga Hridaya.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Shalakya Tantra</t>
+          <t>Sanskrit</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Shalakya deals with?</t>
+          <t>Meaning of 'Vaidya'?</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Heart</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Bones</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>King</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>It deals with Urdhwajatrugata rogas.</t>
+          <t>Vaidya means physician.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Shalya Tantra</t>
+          <t>Shalakya Tantra</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Shalya Tantra deals with?</t>
+          <t>Shalakya deals with?</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Bones</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>Skin</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Shalya Tantra is surgical branch.</t>
+          <t>It deals with Urdhwajatrugata rogas.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>Shalya Tantra</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Shalya Tantra deals with?</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Pediatrics</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Diet</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Surgery</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Shalya Tantra is surgical branch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
           <t>Swasthavritta</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>Dinacharya refers to?</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>Daily routine</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>Night routine</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>Seasonal routine</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G76" t="inlineStr">
         <is>
           <t>Daily routine</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
+      <c r="H76" t="inlineStr">
         <is>
           <t>Dinacharya means daily regimen.</t>
         </is>

</xml_diff>

<commit_message>
Release v1.1.0 - PostgreSQL migration complete
</commit_message>
<xml_diff>
--- a/AIAPGET_Questions.xlsx
+++ b/AIAPGET_Questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,7 +466,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Agadatantra deals with?</t>
+          <t>Agadatantra deals with ?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -592,37 +592,37 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>What is the currently accepted botanical name for the Ayurvedic herb Tagara?</t>
+          <t>WHICH PLANT HAS THIS FLOWERS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Valeriana officinalis</t>
+          <t>RASNA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Valeriana jatamansi</t>
+          <t>ATIVISHA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Valeriana hardwickii</t>
+          <t>TAGARA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Nardostachys jatamansi</t>
+          <t>MUSTA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Valeriana jatamansi</t>
+          <t>TAGARA</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>While historically known as Valeriana wallichii, modern botanical taxonomy recognizes Valeriana jatamansi Jones as the accepted name. Valeriana officinalis is European Valerian, and Nardostachys jatamansi is a completely different plant (Jatamansi/Spikenard).</t>
+          <t>The Flowers: As seen in the top rows, they grow in small, tightly clustered umbels. The individual buds open from a distinct dark pink or purplish color into a soft, pale pinkish-white blossom</t>
         </is>
       </c>
     </row>
@@ -634,205 +634,205 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kaumarabhritya deals with?</t>
+          <t>kaumarabhritya is also called as</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Children</t>
+          <t>bala roga</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Adults</t>
+          <t>kumara vijnana</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Elderly</t>
+          <t>kumara stree vijnana</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>all</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Children</t>
+          <t>bala roga</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>It is pediatrics.</t>
+          <t>refer book</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kaumarabhritya</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>kaumarabhritya is also called as</t>
+          <t>Vata is composed of?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>bala roga</t>
+          <t>Agni</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>kumara vijnana</t>
+          <t>Vayu + Akasha</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>kumara stree vijnana</t>
+          <t>Jala</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>Prithvi</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>bala roga</t>
+          <t>Vayu + Akasha</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>refer book</t>
+          <t>Vata is formed by Vayu and Akasha.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>Kriya Sharira</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Vata is composed of?</t>
+          <t>Pitta is mainly responsible for?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Agni</t>
+          <t>Movement</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Vayu + Akasha</t>
+          <t>Digestion</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Jala</t>
+          <t>Structure</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Prithvi</t>
+          <t>Lubrication</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Vayu + Akasha</t>
+          <t>Digestion</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Vata is formed by Vayu and Akasha.</t>
+          <t>Pitta governs digestion and metabolism.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kriya Sharira</t>
+          <t>Modern Topics</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pitta is mainly responsible for?</t>
+          <t>WHO stands for?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Movement</t>
+          <t>World Health Organization</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Digestion</t>
+          <t>World Human Org</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Structure</t>
+          <t>Health World Org</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Lubrication</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Digestion</t>
+          <t>World Health Organization</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Pitta governs digestion and metabolism.</t>
+          <t>WHO is global health body.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Modern Topics</t>
+          <t>Padartha VIjnana</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>WHO stands for?</t>
+          <t>विवर्त वाद IS ACCEPTE BY</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>World Health Organization</t>
+          <t>जैन</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>World Human Org</t>
+          <t>वैशेषिक</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Health World Org</t>
+          <t>चार्वाक</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>वेदान्त</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>World Health Organization</t>
+          <t>वेदान्त</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>WHO is global health body.</t>
+          <t>SEE BOOK</t>
         </is>
       </c>
     </row>
@@ -844,32 +844,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>विवर्त वाद IS ACCEPTE BY</t>
+          <t>IN सृष्टि उत्पत्ति, नप्रकृति न विकृति IS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>अहंकार</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>पुरुष</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>चार्वाक</t>
+          <t>महत्</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>मनस्</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>पुरुष</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -886,32 +886,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IN सृष्टि उत्पत्ति, नप्रकृति न विकृति IS</t>
+          <t>ACCORDING TO कारिकावलि, THE सामान्य WHICH PERVADES ALL द्रव्य, गुण , कर्म IS CALLED AS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>अहंकार</t>
+          <t>परसामान्य</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>अपरसामान्य</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>महत्</t>
+          <t xml:space="preserve">परापरसामान्य </t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>मनस्</t>
+          <t>विशेषसामन्य</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>परसामान्य</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -928,32 +928,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ACCORDING TO कारिकावलि, THE सामान्य WHICH PERVADES ALL द्रव्य, गुण , कर्म IS CALLED AS</t>
+          <t>THE अभाव WHICH IS BOTH  आदि AND अनन्त IS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>परसामान्य</t>
+          <t>प्राग्भाव</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>अपरसामान्य</t>
+          <t>प्रध्वंसाभाव</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">परापरसामान्य </t>
+          <t>अन्योन्याभाव</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>विशेषसामन्य</t>
+          <t>सर्वाभाव</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>परसामान्य</t>
+          <t>अन्योन्याभाव</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -970,32 +970,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>THE अभाव WHICH IS BOTH  आदि AND अनन्त IS</t>
+          <t>IN अनुमान, परामर्श WILL EVOLVE</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>प्राग्भाव</t>
+          <t>AFTER ESTABLISHMENT OF व्याप्ति</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>प्रध्वंसाभाव</t>
+          <t>BEFORE व्याप्ति</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>अन्योन्याभाव</t>
+          <t>AFTER पक्षधर्मत</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>सर्वाभाव</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>अन्योन्याभाव</t>
+          <t>AFTER पक्षधर्मत</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1012,32 +1012,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IN अनुमान, परामर्श WILL EVOLVE</t>
+          <t>THE STATEMENT, पृथ्वि IS DIFFERENT FROM OTHER भूतs BECAUSE THEY DONT HAVE गन्धगुण IS AN EXAMPLE OF</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AFTER ESTABLISHMENT OF व्याप्ति</t>
+          <t>केवलान्वयि</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BEFORE व्याप्ति</t>
+          <t>केवलव्यतिरेकि</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AFTER पक्षधर्मत</t>
+          <t xml:space="preserve">BOTH </t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>विशेष व्यतिरेकि</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>AFTER पक्षधर्मत</t>
+          <t>केवलव्यतिरेकि</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1054,32 +1054,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>THE STATEMENT, पृथ्वि IS DIFFERENT FROM OTHER भूतs BECAUSE THEY DONT HAVE गन्धगुण IS AN EXAMPLE OF</t>
+          <t>धर्म, अधर्म ARE पदार्थ/DRAVYA ACCORDING TO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>केवलान्वयि</t>
+          <t>सांख्य</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>केवलव्यतिरेकि</t>
+          <t>जैन</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOTH </t>
+          <t>वेदान्त</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>विशेष व्यतिरेकि</t>
+          <t>बौद्ध</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>केवलव्यतिरेकि</t>
+          <t>जैन</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1096,32 +1096,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>धर्म, अधर्म ARE पदार्थ/DRAVYA ACCORDING TO</t>
+          <t>विशिष्टाद्वैत POPULARISED BY</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>सांख्य</t>
+          <t>रामानुजाचार्य</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>शंकराचार्य</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>वेदान्त</t>
+          <t>मध्वाचार्य</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>बौद्ध</t>
+          <t>प्रभाकर</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>जैन</t>
+          <t>रामानुजाचार्य</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1138,32 +1138,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>विशिष्टाद्वैत POPULARISED BY</t>
+          <t>चेष्टा प्रमाण IS ACCEPTED BY</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>रामानुजाचार्य</t>
+          <t>प्रभाकर मीमांस</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>शंकराचार्य</t>
+          <t>पौराणिक</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>मध्वाचार्य</t>
+          <t>तान्त्रिक</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>प्रभाकर</t>
+          <t>मध्व</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>रामानुजाचार्य</t>
+          <t>तान्त्रिक</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1180,32 +1180,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>चेष्टा प्रमाण IS ACCEPTED BY</t>
+          <t>FROM WHICH दर्शन AYURVEDA TAKEN षट् पदार्थ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>प्रभाकर मीमांस</t>
+          <t xml:space="preserve">सांख्य </t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>पौराणिक</t>
+          <t>योग</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>तान्त्रिक</t>
+          <t>न्याय</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>मध्व</t>
+          <t>वैशेषिक</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>तान्त्रिक</t>
+          <t>वैशेषिक</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1222,32 +1222,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FROM WHICH दर्शन AYURVEDA TAKEN षट् पदार्थ</t>
+          <t>ACCORDING TO चरक अतिवाहिक पुरुष IS NOT ASSOCIATED WITH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">सांख्य </t>
+          <t>मन</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>योग</t>
+          <t xml:space="preserve">मन- आकाश       </t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>न्याय</t>
+          <t>इन्द्रिय</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>वैशेषिक</t>
+          <t>इन्द्रिय</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1264,32 +1264,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ACCORDING TO चरक अतिवाहिक पुरुष IS NOT ASSOCIATED WITH</t>
+          <t>षट् पदार्थ ARE CALLED BY चरक AS</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>मन</t>
+          <t>कार्य</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">मन- आकाश       </t>
+          <t>पदार्थ</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>इन्द्रिय</t>
+          <t>कारण</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>विशेष</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>इन्द्रिय</t>
+          <t>कारण</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1306,32 +1306,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>षट् पदार्थ ARE CALLED BY चरक AS</t>
+          <t>WHICH इन्द्रिय प्रत्यक्ष प्रमाण NOT USED TO EXAMINE रोगि</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>कार्य</t>
+          <t>स्पर्शनेन्द्रिय</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>पदार्थ</t>
+          <t xml:space="preserve">चक्षुरेन्द्रिय </t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>रस्नेन्द्रिय</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>विशेष</t>
+          <t>घ्राणेन्द्रिय</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>कारण</t>
+          <t>रस्नेन्द्रिय</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1348,32 +1348,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>WHICH इन्द्रिय प्रत्यक्ष प्रमाण NOT USED TO EXAMINE रोगि</t>
+          <t>यस्य विवरणे शक्ति: IS</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>स्पर्शनेन्द्रिय</t>
+          <t>खर</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">चक्षुरेन्द्रिय </t>
+          <t xml:space="preserve">द्रव </t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>रस्नेन्द्रिय</t>
+          <t xml:space="preserve">सूक्ष्म       </t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>घ्राणेन्द्रिय</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>रस्नेन्द्रिय</t>
+          <t>सूक्ष्म</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1390,32 +1390,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>यस्य विवरणे शक्ति: IS</t>
+          <t>THE ELASTICITY OF RUBBER IS AN EXAMPLE FOR</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>खर</t>
+          <t xml:space="preserve">वेगाख्य संस्कार </t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">द्रव </t>
+          <t>स्थितिस्थापक</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">सूक्ष्म       </t>
+          <t>प्रतिविरुद्ध</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>भावनाख्य संस्कार</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>सूक्ष्म</t>
+          <t>स्थितिस्थापक</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1432,32 +1432,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>THE ELASTICITY OF RUBBER IS AN EXAMPLE FOR</t>
+          <t>FOLLOWING IS NOT THE USE OF काल</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">वेगाख्य संस्कार </t>
+          <t>DRUG ADMINISTRATION</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>स्थितिस्थापक</t>
+          <t>KNOWING DISESE STATUS</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>प्रतिविरुद्ध</t>
+          <t xml:space="preserve">KNOWING SEASONS      </t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>भावनाख्य संस्कार</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>स्थितिस्थापक</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1474,32 +1474,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>FOLLOWING IS NOT THE USE OF काल</t>
+          <t>अविनावभाव सम्बन्ध IS</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DRUG ADMINISTRATION</t>
+          <t>सामान्यतो दॄष्ट अनुमान</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>KNOWING DISESE STATUS</t>
+          <t>अन्वयव्यतिरेकि</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">KNOWING SEASONS      </t>
+          <t>कल्पना</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>व्याप्ति</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>व्याप्ति</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1516,163 +1516,163 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>अविनावभाव सम्बन्ध IS</t>
+          <t>SEE THE IMAGE AND IDENTIFY THE अभाव</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>सामान्यतो दॄष्ट अनुमान</t>
+          <t>प्राग्भाव</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>अन्वयव्यतिरेकि</t>
+          <t>अत्यंतअभाव</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>कल्पना</t>
+          <t>प्रध्वंसाभाव</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>व्याप्ति</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>व्याप्ति</t>
+          <t>प्रध्वंसाभाव</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>SEE BOOK</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Padartha VIjnana</t>
+          <t>Panchakarma</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SEE THE IMAGE AND IDENTIFY THE अभाव</t>
+          <t>Vamana is?</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>प्राग्भाव</t>
+          <t>Emesis</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>अत्यंतअभाव</t>
+          <t>Purgation</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>प्रध्वंसाभाव</t>
+          <t>Enema</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>Nasal therapy</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>प्रध्वंसाभाव</t>
+          <t>Emesis</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Vamana is therapeutic emesis.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Panchakarma</t>
+          <t>Prasooti Tantra &amp; Stree Roga</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Vamana is?</t>
+          <t>Garbhini means?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Emesis</t>
+          <t>Pregnant woman</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Purgation</t>
+          <t>Child</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Enema</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Nasal therapy</t>
+          <t>Nurse</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Emesis</t>
+          <t>Pregnant woman</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Vamana is therapeutic emesis.</t>
+          <t>Garbhini refers to pregnant woman.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Prasooti Tantra &amp; Stree Roga</t>
+          <t>Rachana Sharira</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Garbhini means?</t>
+          <t>Number of bones in adult human body?</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Pregnant woman</t>
+          <t>206</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Child</t>
+          <t>210</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>300</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Nurse</t>
+          <t>180</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Pregnant woman</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Garbhini refers to pregnant woman.</t>
+          <t>Adult human body has 206 bones.</t>
         </is>
       </c>
     </row>
@@ -1684,37 +1684,37 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Number of bones in adult human body?</t>
+          <t>"UDAKADHARA" IS A LAYER OF SKIN ACCORDING TO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>CHARAKA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>SUSHRUTA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>LAGHU VAGBHATA</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>VRUDDHA VAGBHATA</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>CHARAKA</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Adult human body has 206 bones.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
@@ -1726,37 +1726,37 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>"UDAKADHARA" IS A LAYER OF SKIN ACCORDING TO</t>
+          <t>Dwidhatvatmaka Purush includes</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CHARAKA</t>
+          <t>Soumya and Agneya</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SUSHRUTA</t>
+          <t>Shareera and Aatma</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>LAGHU VAGBHATA</t>
+          <t>Raja and Tama</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>VRUDDHA VAGBHATA</t>
+          <t>Mahat and Aahankara</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>CHARAKA</t>
+          <t>Shareera and Aatma</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>PRESENT IN RACHANA BOOKS EXACT WORD NOT IN SAMHITAS</t>
         </is>
       </c>
     </row>
@@ -1768,37 +1768,37 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Dwidhatvatmaka Purush includes</t>
+          <t>Total number of Jaala are</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Soumya and Agneya</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Shareera and Aatma</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Raja and Tama</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Mahat and Aahankara</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Shareera and Aatma</t>
+          <t>16</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>PRESENT IN RACHANA BOOKS EXACT WORD NOT IN SAMHITAS</t>
+          <t>ACCORDING TO SUSHRUTA, VAGBHATA, BHAVAMISHRA, SHARANGADHARA. CHARAKA DIDN’T TOLD</t>
         </is>
       </c>
     </row>
@@ -1810,37 +1810,37 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Total number of Jaala are</t>
+          <t>Which of the following structures are involved in Akshepaka and Danda-Akshepaka?</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>ASTHI SANGHATA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>KURCHA</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>KANDARA</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>SEEMANTHA</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>KANDARA</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>ACCORDING TO SUSHRUTA, VAGBHATA, BHAVAMISHRA, SHARANGADHARA. CHARAKA DIDN’T TOLD</t>
+          <t>REFER SU.NI.1</t>
         </is>
       </c>
     </row>
@@ -1852,37 +1852,37 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Which of the following structures are involved in Akshepaka and Danda-Akshepaka?</t>
+          <t>Dhairya, Chyavana, Priti, Dehabala are said in the context of</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ASTHI SANGHATA</t>
+          <t>Shuddha Aartava</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>KURCHA</t>
+          <t>Shuddha Shukra</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>KANDARA</t>
+          <t>Shukra Functions</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>SEEMANTHA</t>
+          <t>Aartava Functions</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>KANDARA</t>
+          <t>Shukra Functions</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>REFER SU.NI.1</t>
+          <t>KNOW DIFFERENCE BETWEEN KARMA AND GUNA</t>
         </is>
       </c>
     </row>
@@ -1894,37 +1894,37 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dhairya, Chyavana, Priti, Dehabala are said in the context of</t>
+          <t>Sira Vedhya in Dakodara is done 4 Angula left of</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Shuddha Aartava</t>
+          <t>Kurcha</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Shuddha Shukra</t>
+          <t>Sevani</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Shukra Functions</t>
+          <t>Seemantha</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Aartava Functions</t>
+          <t>Asthi sanghata</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Shukra Functions</t>
+          <t>Sevani</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>KNOW DIFFERENCE BETWEEN KARMA AND GUNA</t>
+          <t>REFER SU.SHA.8</t>
         </is>
       </c>
     </row>
@@ -1936,37 +1936,37 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Sira Vedhya in Dakodara is done 4 Angula left of</t>
+          <t>Maternal surface of the Placenta develops from</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Kurcha</t>
+          <t>Decidua Basalis</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Sevani</t>
+          <t>Decidua Capsularis</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Seemantha</t>
+          <t>Chorion Leavae</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Asthi sanghata</t>
+          <t>Chorion Frondosum</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Sevani</t>
+          <t>Decidua Basalis</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>REFER SU.SHA.8</t>
+          <t>MATERNAL COMPONENT ENTIRELY DEVOLOPS FROM THIS WHICH MAKES BASAL PLATE WHICH FACES UTERINE WALL</t>
         </is>
       </c>
     </row>
@@ -1978,37 +1978,37 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Maternal surface of the Placenta develops from</t>
+          <t>Which of the following is a Sesamoid bone?</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Decidua Basalis</t>
+          <t>Palatine</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Decidua Capsularis</t>
+          <t>Mandible</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Chorion Leavae</t>
+          <t>Maxilla</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Chorion Frondosum</t>
+          <t>Patella</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Decidua Basalis</t>
+          <t>Patella</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>MATERNAL COMPONENT ENTIRELY DEVOLOPS FROM THIS WHICH MAKES BASAL PLATE WHICH FACES UTERINE WALL</t>
+          <t>PATELLA IS THE LARGEST SESMOID BONE, WHICH DEVELOPS INSIDE THICK TENDON OF QUADRICEPS FEMORIS</t>
         </is>
       </c>
     </row>
@@ -2020,79 +2020,79 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Which of the following is a Sesamoid bone?</t>
+          <t>Which of the following type of Snayu is present in Parshwa?</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Palatine</t>
+          <t>Prutu</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mandible</t>
+          <t>Sushira</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Maxilla</t>
+          <t>Pratanavati</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Patella</t>
+          <t>Vrutta</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Patella</t>
+          <t>Pratanavati</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>PATELLA IS THE LARGEST SESMOID BONE, WHICH DEVELOPS INSIDE THICK TENDON OF QUADRICEPS FEMORIS</t>
+          <t>REFER SU. SHA.5</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Rachana Sharira</t>
+          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Which of the following type of Snayu is present in Parshwa?</t>
+          <t>Parada is?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Prutu</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Sushira</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Pratanavati</t>
+          <t>Iron</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Vrutta</t>
+          <t>Copper</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Pratanavati</t>
+          <t>Mercury</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>REFER SU. SHA.5</t>
+          <t>Parada refers to mercury.</t>
         </is>
       </c>
     </row>
@@ -2104,163 +2104,163 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Parada is?</t>
+          <t>Mitra panchaka varga dravyas used in which Bhasma pariksha</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Apunarbhava</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Nirutta</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Iron</t>
+          <t>Varitara</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>Rekhapurna</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Mercury</t>
+          <t>Apunarbhava</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Parada refers to mercury.</t>
+          <t>APUNARBHAVA IS A HIGH TEMPERATURE METALLURGICAL REDUCTION TEST BY USING ORGANIC COMPUNDS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Rasashastra &amp; Bhaishajya Kalpana</t>
+          <t>Research Methodology &amp; Statistics</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mitra panchaka varga dravyas used in which Bhasma pariksha</t>
+          <t>Mean is?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Apunarbhava</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Nirutta</t>
+          <t>Median</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Varitara</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Rekhapurna</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Apunarbhava</t>
+          <t>Average</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>APUNARBHAVA IS A HIGH TEMPERATURE METALLURGICAL REDUCTION TEST BY USING ORGANIC COMPUNDS</t>
+          <t>Mean is average.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Research Methodology &amp; Statistics</t>
+          <t>Roganidana</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Mean is?</t>
+          <t>Nidana means?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Median</t>
+          <t>Treatment</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Exercise</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Diagnosis</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Mean is average.</t>
+          <t>Nidana refers to diagnosis.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Roganidana</t>
+          <t>Samhita Adhyayana 1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Nidana means?</t>
+          <t>Charaka Samhita belongs to?</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>Shalya</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Treatment</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>Shalakya</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Exercise</t>
+          <t>Kaumarabhritya</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>Kayachikitsa</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Nidana refers to diagnosis.</t>
+          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
         </is>
       </c>
     </row>
@@ -2272,37 +2272,37 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Charaka Samhita belongs to?</t>
+          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Shalya</t>
+          <t>तैल</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Shalakya</t>
+          <t>वसा</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Kaumarabhritya</t>
+          <t>मज्जा</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Kayachikitsa</t>
+          <t>घृत</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Charaka Samhita mainly deals with Kayachikitsa.</t>
+          <t>REFER BOOK</t>
         </is>
       </c>
     </row>
@@ -2314,32 +2314,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>संस्कारात् सर्वरोगजित् is told for which sneha as per वाग्भट</t>
+          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>तैल</t>
+          <t>शिशिर</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>वसा</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>मज्जा</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>घृत</t>
+          <t>शरद्</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2356,32 +2356,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dosha which will undergo चय in greeshma ritu should be eliminated in which ritu</t>
+          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>शिशिर</t>
+          <t>शब्दकल्पद्रुम</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>तत्वचन्द्रिक</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>न्यायचन्द्रिक</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>शरद्</t>
+          <t>निबन्धसंग्रह</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2398,32 +2398,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>COMMENTARY OF डल्हण ON सुश्रुतसंहिता IS</t>
+          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>शब्दकल्पद्रुम</t>
+          <t>चरक</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>तत्वचन्द्रिक</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>अग्निवेश</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>न्यायचन्द्रिक</t>
+          <t>नागार्जुन</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>निबन्धसंग्रह</t>
+          <t>दॄढबल</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2440,32 +2440,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>प्रतिसंस्कर्त OF चरकसंहिता IS</t>
+          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>चरक</t>
+          <t>इंन्द्र</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>सहस्राक्ष</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>अग्निवेश</t>
+          <t>प्रजापति</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>नागार्जुन</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>दॄढबल</t>
+          <t>a AND B</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2482,32 +2482,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>IN THE ORDER OF आयुर्वेद अवतरण AFTER अश्विनौ WHO WILL COME</t>
+          <t>भिन्नक्रम IS A</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>इंन्द्र</t>
+          <t>तन्त्रयुक्ति</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>सहस्राक्ष</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>प्रजापति</t>
+          <t>BOTH</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>तन्त्रगुण</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>a AND B</t>
+          <t>तन्त्रदोष</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2524,32 +2524,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>भिन्नक्रम IS A</t>
+          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>तन्त्रयुक्ति</t>
+          <t>अध्यायन</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>अध्यापन</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>BOTH</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>तन्त्रगुण</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>तन्त्रदोष</t>
+          <t>तद्विध्यसम्भाष</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2566,32 +2566,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>वाद COMES UNDER WHICH त्रिविदज्ञानोपाय</t>
+          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>अध्यायन</t>
+          <t>34</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>अध्यापन</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>तद्विध्यसम्भाष</t>
+          <t>36</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2608,32 +2608,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>NUMBER OF तन्त्रयुक्ति TOLD BY अरुणदत्त IS</t>
+          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>एकदोषज</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>त्रिदोषज</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>वातज</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>द्विदोषज</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2650,32 +2650,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WHICH TYPE OF प्रकॄति IS निन्ध्य</t>
+          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>एकदोषज</t>
+          <t>अष्टांग हृदय</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>त्रिदोषज</t>
+          <t>सुश्रुत संहिता</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>वातज</t>
+          <t>अष्टांग संग्रह</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>द्विदोषज</t>
+          <t>चरक संहिता</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2692,32 +2692,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>जल्पकल्पतरु IS THE NAME OF COMMENTARY ON</t>
+          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>अष्टांग हृदय</t>
+          <t>पिप्पलि</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>अपमार्ग</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>सुश्रुत संहिता</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>अष्टांग संग्रह</t>
+          <t>नीलिनी</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>चरक संहिता</t>
+          <t>मदनफल</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2734,32 +2734,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS A वामक द्रव्य</t>
+          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>पिप्पलि</t>
+          <t>वसन्त</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>अपमार्ग</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>शरत्</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>नीलिनी</t>
+          <t>वर्षा</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>मदनफल</t>
+          <t>हेमन्त</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2776,32 +2776,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>प्रबल अनल WILL BE THERE IN FOLLOWING ॠतु</t>
+          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>वसन्त</t>
+          <t>NORTH</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>SOUTH</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>शरत्</t>
+          <t>EAST</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>वर्षा</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>हेमन्त</t>
+          <t>WEST</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2818,32 +2818,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>RIVER FLOWING IN WHICH DIRECTION IS CONSIDERED AS पथ्य</t>
+          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>NORTH</t>
+          <t>मधुर</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>SOUTH</t>
+          <t>आम्ल</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>EAST</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>तिक्त</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>WEST</t>
+          <t>लवण</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2860,32 +2860,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ONE OF THE FOLLOWING IS NOT कषाययोनि</t>
+          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>मधुर</t>
+          <t>84</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>आम्ल</t>
+          <t>72</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>तिक्त</t>
+          <t>108</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>लवण</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2902,32 +2902,32 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>TOTAL NUMBER OF धामार्गव AND चतुरङ्गुम FORMULATIONS ARE</t>
+          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>BLUE</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>YELLOW</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>COPPERISH</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2944,32 +2944,32 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>WHAT TYPE OF COLORED LINES YOU CAN SEE IF THERE IS विष IN मधु</t>
+          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>BLUE</t>
+          <t>तिर्यक्दोष</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>YELLOW</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>COPPERISH</t>
+          <t>अनुपस्थितदोश</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>ऊर्ध्वदोष</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>GREEN</t>
+          <t>उपस्थितदोष</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2986,32 +2986,32 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>पञ्चकर्म SHOULD BE CARRIED OUT IN FOLLOWING CONDITION</t>
+          <t>अवपीडक सर्पि IS GIVEN IN</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>तिर्यक्दोष</t>
+          <t>छर्दिवेगधारण</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>पुरिषवेगधारण</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>अनुपस्थितदोश</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>ऊर्ध्वदोष</t>
+          <t>अश्रुवेगधारण</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>उपस्थितदोष</t>
+          <t>मूत्रवेगधारण</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3028,32 +3028,32 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>अवपीडक सर्पि IS GIVEN IN</t>
+          <t>WHICH IS RIGHT</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>छर्दिवेगधारण</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>पुरिषवेगधारण</t>
+          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>अश्रुवेगधारण</t>
+          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>मूत्रवेगधारण</t>
+          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3070,32 +3070,32 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>WHICH IS RIGHT</t>
+          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>हेतोनईर्ष्य , फलेईर्ष्य</t>
+          <t>ABUNDANT AVAILABILIT</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेईर्ष्य</t>
+          <t>SHOULD HAVE MORE PARTS</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनईर्ष्य</t>
+          <t>MULTIPLE COLORS</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>हेतोईर्ष्य, फलेनेर्ष्य</t>
+          <t>MULTIPLE PROPERTY</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3112,32 +3112,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>बहुता IS ONE OF भेषज गुण, WHICH MEANS</t>
+          <t>सुरा IS IDEAL अनुपान FOR</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>स्थूल</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ABUNDANT AVAILABILIT</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>SHOULD HAVE MORE PARTS</t>
+          <t>शोष</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>MULTIPLE COLORS</t>
+          <t>विष</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>MULTIPLE PROPERTY</t>
+          <t>कृश</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3154,32 +3154,32 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>सुरा IS IDEAL अनुपान FOR</t>
+          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>स्थूल</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>कांस्य</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>शोष</t>
+          <t>स्वर्णा</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>विष</t>
+          <t>मुक्ता</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>कृश</t>
+          <t>रजत</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3196,32 +3196,32 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>WHICH ONE OF THE BELOW HAS आम्ल रस</t>
+          <t>वात प्रकोप IS CAUSED BY</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>उष्ण युक्त रूक्ष</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>कांस्य</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>स्वर्णा</t>
+          <t>शीत युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>मुक्ता</t>
+          <t>उष्ण युक्त स्निग्ध</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>रजत</t>
+          <t>शीत युक्त रूक्ष</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3238,32 +3238,32 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>वात प्रकोप IS CAUSED BY</t>
+          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>उष्ण युक्त रूक्ष</t>
+          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>शीत युक्त स्निग्ध</t>
+          <t>कर्ममिथ्यायोग</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>उष्ण युक्त स्निग्ध</t>
+          <t>वाक् मिथ्यायोग</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>शीत युक्त रूक्ष</t>
+          <t>रसनेन्द्रिय मिथ्यायोग</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3280,32 +3280,32 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>VIOLATING  आहारविधि विशेषायतन COMES UNDER</t>
+          <t>दूषिकI  IS मल OF</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>स्पर्शनेन्द्रिय मिथ्यायोग</t>
+          <t>कर्ण</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>नास</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>कर्ममिथ्यायोग</t>
+          <t>आस्य</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>वाक् मिथ्यायोग</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>रसनेन्द्रिय मिथ्यायोग</t>
+          <t>नेत्र</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3317,292 +3317,250 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 1</t>
+          <t>Samhita Adhyayana 2</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>दूषिकI  IS मल OF</t>
+          <t>Sushruta is known for?</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>कर्ण</t>
+          <t>Medicine</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>नास</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>आस्य</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>Toxicology</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>नेत्र</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>REFER BOOK</t>
+          <t>Sushruta is father of surgery.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 2</t>
+          <t>Samhita Adhyayana 3</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Sushruta is known for?</t>
+          <t>Ashtanga Hridaya written by?</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>Charaka</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Sushruta</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Toxicology</t>
+          <t>Kashyapa</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Vagbhata</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Sushruta is father of surgery.</t>
+          <t>Vagbhata authored Ashtanga Hridaya.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Samhita Adhyayana 3</t>
+          <t>Sanskrit</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Ashtanga Hridaya written by?</t>
+          <t>Meaning of 'Vaidya'?</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Charaka</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Sushruta</t>
+          <t>Teacher</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Kashyapa</t>
+          <t>King</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Vagbhata</t>
+          <t>Doctor</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Vagbhata authored Ashtanga Hridaya.</t>
+          <t>Vaidya means physician.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Sanskrit</t>
+          <t>Shalakya Tantra</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Meaning of 'Vaidya'?</t>
+          <t>Shalakya deals with?</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Teacher</t>
+          <t>Heart</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Bones</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>King</t>
+          <t>Skin</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Doctor</t>
+          <t>ENT &amp; Eye</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Vaidya means physician.</t>
+          <t>It deals with Urdhwajatrugata rogas.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Shalakya Tantra</t>
+          <t>Shalya Tantra</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Shalakya deals with?</t>
+          <t>Shalya Tantra deals with?</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Heart</t>
+          <t>Medicine</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Bones</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>ENT &amp; Eye</t>
+          <t>Surgery</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>It deals with Urdhwajatrugata rogas.</t>
+          <t>Shalya Tantra is surgical branch.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Shalya Tantra</t>
+          <t>Swasthavritta</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Shalya Tantra deals with?</t>
+          <t>Dinacharya refers to?</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Daily routine</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Medicine</t>
+          <t>Night routine</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Seasonal routine</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>Daily routine</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
-        <is>
-          <t>Shalya Tantra is surgical branch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Swasthavritta</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Dinacharya refers to?</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Daily routine</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Night routine</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Seasonal routine</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Daily routine</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
         <is>
           <t>Dinacharya means daily regimen.</t>
         </is>

</xml_diff>